<commit_message>
Improve default handling and staff flow regression
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -990,17 +990,17 @@
           <t>change_registered_office_required</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr"/>
+          <t>默认 Auto</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>留空/Auto 时，填写新注册地址即可生成；填 No 则不生成。</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -1042,19 +1042,15 @@
           <t>change_business_activity_required</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D21" s="5" t="inlineStr"/>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>支持主业务和副业务。</t>
+          <t>留空/Auto 时，填写新 SSIC/业务范围即可生成；填 No 则不生成。支持主业务和副业务。</t>
         </is>
       </c>
     </row>
@@ -1170,17 +1166,17 @@
           <t>change_fye_required</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D26" s="5" t="inlineStr"/>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr"/>
+          <t>默认 Auto</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>留空/Auto 时，填写新 FYE 即可生成；填 No 则不生成。</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
@@ -1302,19 +1298,15 @@
           <t>transfer_in_required</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D31" s="5" t="inlineStr"/>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
+          <t>需要时填 Yes</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
         <is>
-          <t>M02 后续接入。</t>
+          <t>转入没有可靠的新值触发项；需要转入时填 Yes。</t>
         </is>
       </c>
     </row>
@@ -1450,19 +1442,15 @@
           <t>annual_review_required</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D36" s="5" t="inlineStr"/>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>年审包后续接入。</t>
+          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
@@ -2403,43 +2391,43 @@
   </mergeCells>
   <dataValidations count="19">
     <dataValidation sqref="D19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"cooperative,non_cooperative"</formula1>
     </dataValidation>
     <dataValidation sqref="D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="A45:A52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="B45:B52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"appoint_director,resign_director,appoint_secretary,resign_secretary"</formula1>
     </dataValidation>
     <dataValidation sqref="E45:E52" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="A56:A63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="C56:C63" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ID type,ID number,Residential address,Email,Phone,Nationality,Name,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="A67:A74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="K67:K74" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"internal_paid_up_basis,acra_paid_up_capital_basis,stamp_duty_higher_of_price_or_nav"</formula1>
@@ -2451,7 +2439,7 @@
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="A78:A85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="M78:M85" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
@@ -2537,19 +2525,15 @@
           <t>annual_review_required</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+      <c r="D4" s="5" t="inlineStr"/>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>选 Yes 才生成</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>这是年审页主开关。</t>
+          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
@@ -3007,7 +2991,7 @@
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"No,Yes"</formula1>
+      <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ordinary_agm,exempt_private_company,dormant_company,manual"</formula1>

</xml_diff>

<commit_message>
Update secretary generator templates and workflow
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -2458,12 +2458,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="2" max="2"/>
+    <col width="31" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
@@ -2720,193 +2720,209 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>财报日期</t>
+          <t>公司活动状态</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Financial statement date</t>
+          <t>Company activity status</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>financial_statement_date</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>company_activity_status</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>默认 FYE</t>
+          <t>默认</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>留空默认财年结束日。</t>
+          <t>Active / Dormant；留空按 Active。</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>董事签字人</t>
+          <t>是否 ACRA 休眠相关公司</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Director signer</t>
+          <t>ACRA dormant relevant company</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>director_signer_name</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr"/>
+          <t>acra_dormant_relevant_company</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>常用</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>留空默认首页董事签字人。</t>
+          <t>Auto / Yes / No；休眠公司会影响是否需要财报。</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>股东/成员签字人</t>
+          <t>资产是否不超过 50 万</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Shareholder signer</t>
+          <t>Total assets under S$500k</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>shareholder_signer_name</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr"/>
+          <t>total_assets_under_500k</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>可空</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>需要股东签署的年审文件使用。</t>
+          <t>Auto / Yes / No；用于判断 dormant AGM exemption 风险。</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>AR 授权签字人</t>
+          <t>是否需要财报</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>AR authorised signer</t>
+          <t>Financial statements required</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>ar_authorized_signer_name</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
+          <t>financial_statements_required</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>默认董事签字人</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Annual Return 授权。</t>
+          <t>Auto / Yes / No；休眠且符合条件时可 No。</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>董事费</t>
+          <t>财报类型</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Directors' fee</t>
+          <t>Financial statements type</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>directors_fee</t>
+          <t>financial_statements_type</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>默认</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>通常 0。</t>
+          <t>Auto / Unaudited / Audited / Dormant no FS / Management accounts。</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>董事薪酬</t>
+          <t>审计/豁免状态</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Directors' remuneration</t>
+          <t>Audit exemption status</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>directors_remuneration</t>
+          <t>audit_exemption_status</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>默认</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>通常 0。</t>
+          <t>Auto / Small company exempt / Audited / Dormant relevant / Manual review。</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Shorter Notice Consent</t>
+          <t>AGM 状态</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Shorter notice consent</t>
+          <t>AGM status</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>shorter_notice_consent</t>
+          <t>agm_status</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
@@ -2916,70 +2932,310 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>默认</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Auto / Yes / No。</t>
+          <t>Auto / Held AGM / Dispensed with AGM / Exempt from AGM / Written resolutions。</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Management Representation Letter</t>
+          <t>IRAS 税务状态</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>MRL</t>
+          <t>IRAS tax status</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>management_rep_letter</t>
+          <t>iras_tax_status</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Auto</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>默认</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Yes / No。</t>
+          <t>Auto / Active / Dormant / Dormant waiver granted / Manual review；只作复核提醒。</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>财报日期</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Remarks</t>
+          <t>Financial statement date</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>remarks</t>
+          <t>financial_statement_date</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr">
         <is>
+          <t>默认 FYE</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>留空默认财年结束日。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>董事签字人</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Director signer</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>director_signer_name</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>常用</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>留空默认首页董事签字人。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>股东/成员签字人</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Shareholder signer</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>shareholder_signer_name</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>需要股东签署的年审文件使用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>AR 授权签字人</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>AR authorised signer</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>ar_authorized_signer_name</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>默认董事签字人</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>Annual Return 授权。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>董事费</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Directors' fee</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>directors_fee</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>默认</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>通常 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>董事薪酬</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Directors' remuneration</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>directors_remuneration</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>默认</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>通常 0。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Shorter Notice Consent</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Shorter notice consent</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>shorter_notice_consent</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Auto</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>默认</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>Auto / Yes / No。</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Management Representation Letter</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>MRL</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>management_rep_letter</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>默认</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>Yes / No。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>remarks</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>可空</t>
+        </is>
+      </c>
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>特殊情况写这里。</t>
         </is>
@@ -2989,17 +3245,44 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="13">
     <dataValidation sqref="D4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ordinary_agm,exempt_private_company,dormant_company,manual"</formula1>
+      <formula1>"ordinary_agm,exempt_private_company,dormant_company,written_resolutions,manual"</formula1>
     </dataValidation>
     <dataValidation sqref="D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"non_dormant,dormant,unaudited,audited"</formula1>
+      <formula1>"non_dormant,dormant,unaudited,audited,manual"</formula1>
     </dataValidation>
-    <dataValidation sqref="D17:D18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Active,Dormant"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Unaudited,Audited,Dormant no FS,Management accounts,Not applicable"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Small company exempt,Audited,Dormant relevant,Manual review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Held AGM,Dispensed with AGM,Exempt from AGM,Written resolutions,Manual review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Active,Dormant,Dormant waiver granted,Manual review"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
+    <dataValidation sqref="D26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Advance secretary document generator
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -84,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -92,11 +92,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -117,6 +131,25 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,7 +540,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>P2 一页式快速业务单 - 少填字段先生成文件</t>
         </is>
@@ -515,1052 +548,1048 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>field_key</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>填写内容 / Value</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>公司名称</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Company name</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr"/>
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>所有文件都会用。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>UEN / 注册号</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>UEN</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>uen</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>现有公司变更建议填写。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>当前注册地址</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>Current registered office</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>registered_office_address</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>多数文件会用；地址变更时作为旧地址。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>当前总股数</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>Current total shares</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>total_issued_shares</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr"/>
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>用于增资配股后资本推导；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>当前已发行股本</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Current issued share capital</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>issued_share_capital</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>对应 ACRA issued share capital；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>当前实缴资本</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Current paid-up share capital</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>paid_up_capital</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr"/>
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>对应 ACRA paid-up share capital；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>币种</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>SGD</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>通常 SGD；如 USD 等请填写。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>文件日期</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Document date</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>default_document_date</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr"/>
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>DD/MM/YYYY；留空后续可由网页补当天。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>M01 directors to sign</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>M01 director signer names</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>director_signer_names</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr"/>
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Enter all current directors for M01. One per line, comma, or semicolon.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>股东/成员签字人姓名</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Member/shareholder signer names</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>member_signer_names</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr"/>
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>转入建议填</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>M02 股东/成员签署处使用；多人可换行、逗号或分号分隔。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>客户方签字人姓名</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Client signer name</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>client_signatory_name</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr"/>
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>交接信签字人；留空默认用第一个股东/成员签字人。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>业务单编号</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Business order ID</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>business_order_id</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>后台预留。</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Source type</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>AI / BizFile / Excel / Manual。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>来源文件编号</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>Source file ID</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>source_file_id</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr"/>
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>可填 BizFile 或旧表文件名。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>经办人</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>prepared_by</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr"/>
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>内部记录。</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>是否变更注册地址</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Change registered office</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>change_registered_office_required</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新注册地址即可生成；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>新注册地址</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>New registered office</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>new_registered_office_address</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>地址变更时填</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr"/>
+      <c r="F20" s="13" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>是否变更营业范围</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Change business activity</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>change_business_activity_required</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新 SSIC/业务范围即可生成；填 No 则不生成。支持主业务和副业务。</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>新主 SSIC</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>New primary SSIC</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>new_primary_ssic</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr"/>
+      <c r="F22" s="13" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>新主营业范围</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>New primary activity</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>new_primary_activity</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr"/>
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>营业范围变更时填</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr"/>
+      <c r="F23" s="13" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>新副 SSIC</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>New secondary SSIC</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>new_secondary_ssic</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr"/>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr"/>
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr"/>
+      <c r="F24" s="13" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>新副营业范围</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>New secondary activity</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>new_secondary_activity</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr"/>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr"/>
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr"/>
+      <c r="F25" s="13" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>是否变更 FYE</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Change FYE</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>change_fye_required</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr"/>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr"/>
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新 FYE 即可生成；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>旧 FYE</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Old FYE</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>old_fye</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>FYE 变更时填</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>新 FYE</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>New FYE</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>new_fye</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr"/>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="D28" s="12" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr">
         <is>
           <t>FYE 变更时填</t>
         </is>
       </c>
-      <c r="F28" s="6" t="inlineStr">
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="10" t="inlineStr">
         <is>
           <t>下个账期开始</t>
         </is>
       </c>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" s="10" t="inlineStr">
         <is>
           <t>Next accounts period start</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>next_accounts_period_start</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr"/>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="D29" s="12" t="inlineStr"/>
+      <c r="E29" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr"/>
+      <c r="F29" s="13" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>下个账期结束</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>Next accounts period end</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>next_accounts_period_end</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr"/>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="D30" s="12" t="inlineStr"/>
+      <c r="E30" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F30" s="6" t="inlineStr"/>
+      <c r="F30" s="13" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>是否转入秘书公司</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="10" t="inlineStr">
         <is>
           <t>Transfer-in required</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>transfer_in_required</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr"/>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="D31" s="12" t="inlineStr"/>
+      <c r="E31" s="10" t="inlineStr">
         <is>
           <t>需要时填 Yes</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>转入没有可靠的新值触发项；需要转入时填 Yes。</t>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>转入需要时填 Yes；M01 正常出，M02 一律兜底。</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>转入模式</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>Transfer-in mode</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>transfer_in_mode</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>cooperative</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="D32" s="12" t="inlineStr"/>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>内部预留</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="inlineStr">
+        <is>
+          <t>通常留空；系统不再要求区分配合/不配合。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>旧秘书公司</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t>Old secretary firm</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>old_secretary_company</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr"/>
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F32" s="6" t="inlineStr">
-        <is>
-          <t>cooperative / non_cooperative。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>旧秘书公司</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>Old secretary firm</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>old_secretary_company</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr"/>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>新秘书公司</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>New secretary firm</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>new_secretary_company</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>RSIN GROUP PTE. LTD.</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
-        <is>
-          <t>新秘书公司</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>New secretary firm</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>new_secretary_company</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>RSIN GROUP PTE. LTD.</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="F34" s="13" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>是否出辞职信</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t>Generate resignation letter</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>generate_resignation_letter</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="3" t="inlineStr">
-        <is>
-          <t>是否出辞职信</t>
-        </is>
-      </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>Generate resignation letter</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>generate_resignation_letter</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>只有需要旧人员单独签辞职信时填 Yes；一般留 No。</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>是否做年审</t>
+        </is>
+      </c>
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>Annual review required</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>annual_review_required</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr"/>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>默认 Auto</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>年审 FYE</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Annual review FYE</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>fye_date</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr"/>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>年审时填</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>DD/MM/YYYY。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>AGM 日期</t>
+        </is>
+      </c>
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>AGM date</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>agm_date</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr"/>
+      <c r="E38" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>不配合转入通常 No。</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
-        <is>
-          <t>是否做年审</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>Annual review required</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>annual_review_required</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr"/>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>默认 Auto</t>
-        </is>
-      </c>
-      <c r="F36" s="6" t="inlineStr">
-        <is>
-          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>年审 FYE</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>Annual review FYE</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>fye_date</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr"/>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>年审时填</t>
-        </is>
-      </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="F38" s="13" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>AGM 日期</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>AGM date</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>agm_date</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr"/>
-      <c r="E38" s="3" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>年审备注</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>Annual review remarks</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>annual_review_remarks</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr"/>
+      <c r="E39" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F38" s="6" t="inlineStr">
-        <is>
-          <t>DD/MM/YYYY。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>年审备注</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>Annual review remarks</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>annual_review_remarks</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr"/>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>复杂情况写这里；详细字段可填“快速年审”页。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr"/>
+      <c r="E40" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
-        <is>
-          <t>复杂情况写这里；详细字段可填“快速年审”页。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>备注</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr"/>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>可空</t>
-        </is>
-      </c>
-      <c r="F40" s="6" t="inlineStr">
+      <c r="F40" s="13" t="inlineStr">
         <is>
           <t>内部备注，不进正式文件。</t>
         </is>
@@ -1569,44 +1598,44 @@
     <row r="41"/>
     <row r="42"/>
     <row r="43">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>人员任免</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" s="9" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>动作
 action_type</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" s="9" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E44" s="9" t="inlineStr">
         <is>
           <t>是否出辞职信
 resignation_letter</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1614,115 +1643,115 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr"/>
-      <c r="B45" s="5" t="inlineStr"/>
-      <c r="C45" s="5" t="inlineStr"/>
-      <c r="D45" s="5" t="inlineStr"/>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="A45" s="12" t="inlineStr"/>
+      <c r="B45" s="12" t="inlineStr"/>
+      <c r="C45" s="12" t="inlineStr"/>
+      <c r="D45" s="12" t="inlineStr"/>
+      <c r="E45" s="12" t="inlineStr"/>
+      <c r="F45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="5" t="inlineStr"/>
-      <c r="B46" s="5" t="inlineStr"/>
-      <c r="C46" s="5" t="inlineStr"/>
-      <c r="D46" s="5" t="inlineStr"/>
-      <c r="E46" s="5" t="inlineStr"/>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="A46" s="12" t="inlineStr"/>
+      <c r="B46" s="12" t="inlineStr"/>
+      <c r="C46" s="12" t="inlineStr"/>
+      <c r="D46" s="12" t="inlineStr"/>
+      <c r="E46" s="12" t="inlineStr"/>
+      <c r="F46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="5" t="inlineStr"/>
-      <c r="B47" s="5" t="inlineStr"/>
-      <c r="C47" s="5" t="inlineStr"/>
-      <c r="D47" s="5" t="inlineStr"/>
-      <c r="E47" s="5" t="inlineStr"/>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="A47" s="12" t="inlineStr"/>
+      <c r="B47" s="12" t="inlineStr"/>
+      <c r="C47" s="12" t="inlineStr"/>
+      <c r="D47" s="12" t="inlineStr"/>
+      <c r="E47" s="12" t="inlineStr"/>
+      <c r="F47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="5" t="inlineStr"/>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="5" t="inlineStr"/>
+      <c r="A48" s="12" t="inlineStr"/>
+      <c r="B48" s="12" t="inlineStr"/>
+      <c r="C48" s="12" t="inlineStr"/>
+      <c r="D48" s="12" t="inlineStr"/>
+      <c r="E48" s="12" t="inlineStr"/>
+      <c r="F48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="5" t="inlineStr"/>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
-      <c r="D49" s="5" t="inlineStr"/>
-      <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="A49" s="12" t="inlineStr"/>
+      <c r="B49" s="12" t="inlineStr"/>
+      <c r="C49" s="12" t="inlineStr"/>
+      <c r="D49" s="12" t="inlineStr"/>
+      <c r="E49" s="12" t="inlineStr"/>
+      <c r="F49" s="12" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="5" t="inlineStr"/>
-      <c r="B50" s="5" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="A50" s="12" t="inlineStr"/>
+      <c r="B50" s="12" t="inlineStr"/>
+      <c r="C50" s="12" t="inlineStr"/>
+      <c r="D50" s="12" t="inlineStr"/>
+      <c r="E50" s="12" t="inlineStr"/>
+      <c r="F50" s="12" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr"/>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="5" t="inlineStr"/>
-      <c r="D51" s="5" t="inlineStr"/>
-      <c r="E51" s="5" t="inlineStr"/>
-      <c r="F51" s="5" t="inlineStr"/>
+      <c r="A51" s="12" t="inlineStr"/>
+      <c r="B51" s="12" t="inlineStr"/>
+      <c r="C51" s="12" t="inlineStr"/>
+      <c r="D51" s="12" t="inlineStr"/>
+      <c r="E51" s="12" t="inlineStr"/>
+      <c r="F51" s="12" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="5" t="inlineStr"/>
-      <c r="B52" s="5" t="inlineStr"/>
-      <c r="C52" s="5" t="inlineStr"/>
-      <c r="D52" s="5" t="inlineStr"/>
-      <c r="E52" s="5" t="inlineStr"/>
-      <c r="F52" s="5" t="inlineStr"/>
+      <c r="A52" s="12" t="inlineStr"/>
+      <c r="B52" s="12" t="inlineStr"/>
+      <c r="C52" s="12" t="inlineStr"/>
+      <c r="D52" s="12" t="inlineStr"/>
+      <c r="E52" s="12" t="inlineStr"/>
+      <c r="F52" s="12" t="inlineStr"/>
     </row>
     <row r="53"/>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+      <c r="A54" s="14" t="inlineStr">
         <is>
           <t>个人资料变更</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
+      <c r="A55" s="9" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B55" s="2" t="inlineStr">
+      <c r="B55" s="9" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="C55" s="2" t="inlineStr">
+      <c r="C55" s="9" t="inlineStr">
         <is>
           <t>变更字段
 field_label</t>
         </is>
       </c>
-      <c r="D55" s="2" t="inlineStr">
+      <c r="D55" s="9" t="inlineStr">
         <is>
           <t>原资料
 old_value</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
+      <c r="E55" s="9" t="inlineStr">
         <is>
           <t>新资料
 new_value</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="G55" s="2" t="inlineStr">
+      <c r="G55" s="9" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1730,195 +1759,195 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="5" t="inlineStr"/>
-      <c r="B56" s="5" t="inlineStr"/>
-      <c r="C56" s="5" t="inlineStr"/>
-      <c r="D56" s="5" t="inlineStr"/>
-      <c r="E56" s="5" t="inlineStr"/>
-      <c r="F56" s="5" t="inlineStr"/>
-      <c r="G56" s="5" t="inlineStr"/>
+      <c r="A56" s="12" t="inlineStr"/>
+      <c r="B56" s="12" t="inlineStr"/>
+      <c r="C56" s="12" t="inlineStr"/>
+      <c r="D56" s="12" t="inlineStr"/>
+      <c r="E56" s="12" t="inlineStr"/>
+      <c r="F56" s="12" t="inlineStr"/>
+      <c r="G56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="5" t="inlineStr"/>
-      <c r="B57" s="5" t="inlineStr"/>
-      <c r="C57" s="5" t="inlineStr"/>
-      <c r="D57" s="5" t="inlineStr"/>
-      <c r="E57" s="5" t="inlineStr"/>
-      <c r="F57" s="5" t="inlineStr"/>
-      <c r="G57" s="5" t="inlineStr"/>
+      <c r="A57" s="12" t="inlineStr"/>
+      <c r="B57" s="12" t="inlineStr"/>
+      <c r="C57" s="12" t="inlineStr"/>
+      <c r="D57" s="12" t="inlineStr"/>
+      <c r="E57" s="12" t="inlineStr"/>
+      <c r="F57" s="12" t="inlineStr"/>
+      <c r="G57" s="12" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="5" t="inlineStr"/>
-      <c r="B58" s="5" t="inlineStr"/>
-      <c r="C58" s="5" t="inlineStr"/>
-      <c r="D58" s="5" t="inlineStr"/>
-      <c r="E58" s="5" t="inlineStr"/>
-      <c r="F58" s="5" t="inlineStr"/>
-      <c r="G58" s="5" t="inlineStr"/>
+      <c r="A58" s="12" t="inlineStr"/>
+      <c r="B58" s="12" t="inlineStr"/>
+      <c r="C58" s="12" t="inlineStr"/>
+      <c r="D58" s="12" t="inlineStr"/>
+      <c r="E58" s="12" t="inlineStr"/>
+      <c r="F58" s="12" t="inlineStr"/>
+      <c r="G58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="5" t="inlineStr"/>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="5" t="inlineStr"/>
-      <c r="D59" s="5" t="inlineStr"/>
-      <c r="E59" s="5" t="inlineStr"/>
-      <c r="F59" s="5" t="inlineStr"/>
-      <c r="G59" s="5" t="inlineStr"/>
+      <c r="A59" s="12" t="inlineStr"/>
+      <c r="B59" s="12" t="inlineStr"/>
+      <c r="C59" s="12" t="inlineStr"/>
+      <c r="D59" s="12" t="inlineStr"/>
+      <c r="E59" s="12" t="inlineStr"/>
+      <c r="F59" s="12" t="inlineStr"/>
+      <c r="G59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="5" t="inlineStr"/>
-      <c r="B60" s="5" t="inlineStr"/>
-      <c r="C60" s="5" t="inlineStr"/>
-      <c r="D60" s="5" t="inlineStr"/>
-      <c r="E60" s="5" t="inlineStr"/>
-      <c r="F60" s="5" t="inlineStr"/>
-      <c r="G60" s="5" t="inlineStr"/>
+      <c r="A60" s="12" t="inlineStr"/>
+      <c r="B60" s="12" t="inlineStr"/>
+      <c r="C60" s="12" t="inlineStr"/>
+      <c r="D60" s="12" t="inlineStr"/>
+      <c r="E60" s="12" t="inlineStr"/>
+      <c r="F60" s="12" t="inlineStr"/>
+      <c r="G60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="5" t="inlineStr"/>
-      <c r="B61" s="5" t="inlineStr"/>
-      <c r="C61" s="5" t="inlineStr"/>
-      <c r="D61" s="5" t="inlineStr"/>
-      <c r="E61" s="5" t="inlineStr"/>
-      <c r="F61" s="5" t="inlineStr"/>
-      <c r="G61" s="5" t="inlineStr"/>
+      <c r="A61" s="12" t="inlineStr"/>
+      <c r="B61" s="12" t="inlineStr"/>
+      <c r="C61" s="12" t="inlineStr"/>
+      <c r="D61" s="12" t="inlineStr"/>
+      <c r="E61" s="12" t="inlineStr"/>
+      <c r="F61" s="12" t="inlineStr"/>
+      <c r="G61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="inlineStr"/>
-      <c r="B62" s="5" t="inlineStr"/>
-      <c r="C62" s="5" t="inlineStr"/>
-      <c r="D62" s="5" t="inlineStr"/>
-      <c r="E62" s="5" t="inlineStr"/>
-      <c r="F62" s="5" t="inlineStr"/>
-      <c r="G62" s="5" t="inlineStr"/>
+      <c r="A62" s="12" t="inlineStr"/>
+      <c r="B62" s="12" t="inlineStr"/>
+      <c r="C62" s="12" t="inlineStr"/>
+      <c r="D62" s="12" t="inlineStr"/>
+      <c r="E62" s="12" t="inlineStr"/>
+      <c r="F62" s="12" t="inlineStr"/>
+      <c r="G62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="5" t="inlineStr"/>
-      <c r="B63" s="5" t="inlineStr"/>
-      <c r="C63" s="5" t="inlineStr"/>
-      <c r="D63" s="5" t="inlineStr"/>
-      <c r="E63" s="5" t="inlineStr"/>
-      <c r="F63" s="5" t="inlineStr"/>
-      <c r="G63" s="5" t="inlineStr"/>
+      <c r="A63" s="12" t="inlineStr"/>
+      <c r="B63" s="12" t="inlineStr"/>
+      <c r="C63" s="12" t="inlineStr"/>
+      <c r="D63" s="12" t="inlineStr"/>
+      <c r="E63" s="12" t="inlineStr"/>
+      <c r="F63" s="12" t="inlineStr"/>
+      <c r="G63" s="12" t="inlineStr"/>
     </row>
     <row r="64"/>
     <row r="65">
-      <c r="A65" s="7" t="inlineStr">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>股份转让</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="9" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="9" t="inlineStr">
         <is>
           <t>转让人
 transferor_name</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="9" t="inlineStr">
         <is>
           <t>转让人证件/注册号
 transferor_id_number</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="D66" s="9" t="inlineStr">
         <is>
           <t>转让人地址
 transferor_address</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="9" t="inlineStr">
         <is>
           <t>受让人
 transferee_name</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr">
+      <c r="F66" s="9" t="inlineStr">
         <is>
           <t>受让人证件/注册号
 transferee_id_number</t>
         </is>
       </c>
-      <c r="G66" s="2" t="inlineStr">
+      <c r="G66" s="9" t="inlineStr">
         <is>
           <t>受让人地址
 transferee_address</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
+      <c r="H66" s="9" t="inlineStr">
         <is>
           <t>转让股数
 shares_transferred</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr">
+      <c r="I66" s="9" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="J66" s="2" t="inlineStr">
+      <c r="J66" s="9" t="inlineStr">
         <is>
           <t>转让日期
 transfer_date</t>
         </is>
       </c>
-      <c r="K66" s="2" t="inlineStr">
+      <c r="K66" s="9" t="inlineStr">
         <is>
           <t>对价口径
 consideration_basis</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
+      <c r="L66" s="9" t="inlineStr">
         <is>
           <t>对价金额
 consideration_amount</t>
         </is>
       </c>
-      <c r="M66" s="2" t="inlineStr">
+      <c r="M66" s="9" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="N66" s="2" t="inlineStr">
+      <c r="N66" s="9" t="inlineStr">
         <is>
           <t>旧证书号
 old_certificate_no</t>
         </is>
       </c>
-      <c r="O66" s="2" t="inlineStr">
+      <c r="O66" s="9" t="inlineStr">
         <is>
           <t>新证书号
 new_certificate_no</t>
         </is>
       </c>
-      <c r="P66" s="2" t="inlineStr">
+      <c r="P66" s="9" t="inlineStr">
         <is>
           <t>转让人剩余股数
 transferor_remaining_shares</t>
         </is>
       </c>
-      <c r="Q66" s="2" t="inlineStr">
+      <c r="Q66" s="9" t="inlineStr">
         <is>
           <t>是否生成新证书
 generate_new_certificate</t>
         </is>
       </c>
-      <c r="R66" s="2" t="inlineStr">
+      <c r="R66" s="9" t="inlineStr">
         <is>
           <t>印花税复核
 stamp_duty_review</t>
         </is>
       </c>
-      <c r="S66" s="2" t="inlineStr">
+      <c r="S66" s="9" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1926,291 +1955,291 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="5" t="inlineStr"/>
-      <c r="B67" s="5" t="inlineStr"/>
-      <c r="C67" s="5" t="inlineStr"/>
-      <c r="D67" s="5" t="inlineStr"/>
-      <c r="E67" s="5" t="inlineStr"/>
-      <c r="F67" s="5" t="inlineStr"/>
-      <c r="G67" s="5" t="inlineStr"/>
-      <c r="H67" s="5" t="inlineStr"/>
-      <c r="I67" s="5" t="inlineStr"/>
-      <c r="J67" s="5" t="inlineStr"/>
-      <c r="K67" s="5" t="inlineStr"/>
-      <c r="L67" s="5" t="inlineStr"/>
-      <c r="M67" s="5" t="inlineStr"/>
-      <c r="N67" s="5" t="inlineStr"/>
-      <c r="O67" s="5" t="inlineStr"/>
-      <c r="P67" s="5" t="inlineStr"/>
-      <c r="Q67" s="5" t="inlineStr"/>
-      <c r="R67" s="5" t="inlineStr"/>
-      <c r="S67" s="5" t="inlineStr"/>
+      <c r="A67" s="12" t="inlineStr"/>
+      <c r="B67" s="12" t="inlineStr"/>
+      <c r="C67" s="12" t="inlineStr"/>
+      <c r="D67" s="12" t="inlineStr"/>
+      <c r="E67" s="12" t="inlineStr"/>
+      <c r="F67" s="12" t="inlineStr"/>
+      <c r="G67" s="12" t="inlineStr"/>
+      <c r="H67" s="12" t="inlineStr"/>
+      <c r="I67" s="12" t="inlineStr"/>
+      <c r="J67" s="12" t="inlineStr"/>
+      <c r="K67" s="12" t="inlineStr"/>
+      <c r="L67" s="12" t="inlineStr"/>
+      <c r="M67" s="12" t="inlineStr"/>
+      <c r="N67" s="12" t="inlineStr"/>
+      <c r="O67" s="12" t="inlineStr"/>
+      <c r="P67" s="12" t="inlineStr"/>
+      <c r="Q67" s="12" t="inlineStr"/>
+      <c r="R67" s="12" t="inlineStr"/>
+      <c r="S67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="inlineStr"/>
-      <c r="B68" s="5" t="inlineStr"/>
-      <c r="C68" s="5" t="inlineStr"/>
-      <c r="D68" s="5" t="inlineStr"/>
-      <c r="E68" s="5" t="inlineStr"/>
-      <c r="F68" s="5" t="inlineStr"/>
-      <c r="G68" s="5" t="inlineStr"/>
-      <c r="H68" s="5" t="inlineStr"/>
-      <c r="I68" s="5" t="inlineStr"/>
-      <c r="J68" s="5" t="inlineStr"/>
-      <c r="K68" s="5" t="inlineStr"/>
-      <c r="L68" s="5" t="inlineStr"/>
-      <c r="M68" s="5" t="inlineStr"/>
-      <c r="N68" s="5" t="inlineStr"/>
-      <c r="O68" s="5" t="inlineStr"/>
-      <c r="P68" s="5" t="inlineStr"/>
-      <c r="Q68" s="5" t="inlineStr"/>
-      <c r="R68" s="5" t="inlineStr"/>
-      <c r="S68" s="5" t="inlineStr"/>
+      <c r="A68" s="12" t="inlineStr"/>
+      <c r="B68" s="12" t="inlineStr"/>
+      <c r="C68" s="12" t="inlineStr"/>
+      <c r="D68" s="12" t="inlineStr"/>
+      <c r="E68" s="12" t="inlineStr"/>
+      <c r="F68" s="12" t="inlineStr"/>
+      <c r="G68" s="12" t="inlineStr"/>
+      <c r="H68" s="12" t="inlineStr"/>
+      <c r="I68" s="12" t="inlineStr"/>
+      <c r="J68" s="12" t="inlineStr"/>
+      <c r="K68" s="12" t="inlineStr"/>
+      <c r="L68" s="12" t="inlineStr"/>
+      <c r="M68" s="12" t="inlineStr"/>
+      <c r="N68" s="12" t="inlineStr"/>
+      <c r="O68" s="12" t="inlineStr"/>
+      <c r="P68" s="12" t="inlineStr"/>
+      <c r="Q68" s="12" t="inlineStr"/>
+      <c r="R68" s="12" t="inlineStr"/>
+      <c r="S68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="5" t="inlineStr"/>
-      <c r="B69" s="5" t="inlineStr"/>
-      <c r="C69" s="5" t="inlineStr"/>
-      <c r="D69" s="5" t="inlineStr"/>
-      <c r="E69" s="5" t="inlineStr"/>
-      <c r="F69" s="5" t="inlineStr"/>
-      <c r="G69" s="5" t="inlineStr"/>
-      <c r="H69" s="5" t="inlineStr"/>
-      <c r="I69" s="5" t="inlineStr"/>
-      <c r="J69" s="5" t="inlineStr"/>
-      <c r="K69" s="5" t="inlineStr"/>
-      <c r="L69" s="5" t="inlineStr"/>
-      <c r="M69" s="5" t="inlineStr"/>
-      <c r="N69" s="5" t="inlineStr"/>
-      <c r="O69" s="5" t="inlineStr"/>
-      <c r="P69" s="5" t="inlineStr"/>
-      <c r="Q69" s="5" t="inlineStr"/>
-      <c r="R69" s="5" t="inlineStr"/>
-      <c r="S69" s="5" t="inlineStr"/>
+      <c r="A69" s="12" t="inlineStr"/>
+      <c r="B69" s="12" t="inlineStr"/>
+      <c r="C69" s="12" t="inlineStr"/>
+      <c r="D69" s="12" t="inlineStr"/>
+      <c r="E69" s="12" t="inlineStr"/>
+      <c r="F69" s="12" t="inlineStr"/>
+      <c r="G69" s="12" t="inlineStr"/>
+      <c r="H69" s="12" t="inlineStr"/>
+      <c r="I69" s="12" t="inlineStr"/>
+      <c r="J69" s="12" t="inlineStr"/>
+      <c r="K69" s="12" t="inlineStr"/>
+      <c r="L69" s="12" t="inlineStr"/>
+      <c r="M69" s="12" t="inlineStr"/>
+      <c r="N69" s="12" t="inlineStr"/>
+      <c r="O69" s="12" t="inlineStr"/>
+      <c r="P69" s="12" t="inlineStr"/>
+      <c r="Q69" s="12" t="inlineStr"/>
+      <c r="R69" s="12" t="inlineStr"/>
+      <c r="S69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="5" t="inlineStr"/>
-      <c r="B70" s="5" t="inlineStr"/>
-      <c r="C70" s="5" t="inlineStr"/>
-      <c r="D70" s="5" t="inlineStr"/>
-      <c r="E70" s="5" t="inlineStr"/>
-      <c r="F70" s="5" t="inlineStr"/>
-      <c r="G70" s="5" t="inlineStr"/>
-      <c r="H70" s="5" t="inlineStr"/>
-      <c r="I70" s="5" t="inlineStr"/>
-      <c r="J70" s="5" t="inlineStr"/>
-      <c r="K70" s="5" t="inlineStr"/>
-      <c r="L70" s="5" t="inlineStr"/>
-      <c r="M70" s="5" t="inlineStr"/>
-      <c r="N70" s="5" t="inlineStr"/>
-      <c r="O70" s="5" t="inlineStr"/>
-      <c r="P70" s="5" t="inlineStr"/>
-      <c r="Q70" s="5" t="inlineStr"/>
-      <c r="R70" s="5" t="inlineStr"/>
-      <c r="S70" s="5" t="inlineStr"/>
+      <c r="A70" s="12" t="inlineStr"/>
+      <c r="B70" s="12" t="inlineStr"/>
+      <c r="C70" s="12" t="inlineStr"/>
+      <c r="D70" s="12" t="inlineStr"/>
+      <c r="E70" s="12" t="inlineStr"/>
+      <c r="F70" s="12" t="inlineStr"/>
+      <c r="G70" s="12" t="inlineStr"/>
+      <c r="H70" s="12" t="inlineStr"/>
+      <c r="I70" s="12" t="inlineStr"/>
+      <c r="J70" s="12" t="inlineStr"/>
+      <c r="K70" s="12" t="inlineStr"/>
+      <c r="L70" s="12" t="inlineStr"/>
+      <c r="M70" s="12" t="inlineStr"/>
+      <c r="N70" s="12" t="inlineStr"/>
+      <c r="O70" s="12" t="inlineStr"/>
+      <c r="P70" s="12" t="inlineStr"/>
+      <c r="Q70" s="12" t="inlineStr"/>
+      <c r="R70" s="12" t="inlineStr"/>
+      <c r="S70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="5" t="inlineStr"/>
-      <c r="B71" s="5" t="inlineStr"/>
-      <c r="C71" s="5" t="inlineStr"/>
-      <c r="D71" s="5" t="inlineStr"/>
-      <c r="E71" s="5" t="inlineStr"/>
-      <c r="F71" s="5" t="inlineStr"/>
-      <c r="G71" s="5" t="inlineStr"/>
-      <c r="H71" s="5" t="inlineStr"/>
-      <c r="I71" s="5" t="inlineStr"/>
-      <c r="J71" s="5" t="inlineStr"/>
-      <c r="K71" s="5" t="inlineStr"/>
-      <c r="L71" s="5" t="inlineStr"/>
-      <c r="M71" s="5" t="inlineStr"/>
-      <c r="N71" s="5" t="inlineStr"/>
-      <c r="O71" s="5" t="inlineStr"/>
-      <c r="P71" s="5" t="inlineStr"/>
-      <c r="Q71" s="5" t="inlineStr"/>
-      <c r="R71" s="5" t="inlineStr"/>
-      <c r="S71" s="5" t="inlineStr"/>
+      <c r="A71" s="12" t="inlineStr"/>
+      <c r="B71" s="12" t="inlineStr"/>
+      <c r="C71" s="12" t="inlineStr"/>
+      <c r="D71" s="12" t="inlineStr"/>
+      <c r="E71" s="12" t="inlineStr"/>
+      <c r="F71" s="12" t="inlineStr"/>
+      <c r="G71" s="12" t="inlineStr"/>
+      <c r="H71" s="12" t="inlineStr"/>
+      <c r="I71" s="12" t="inlineStr"/>
+      <c r="J71" s="12" t="inlineStr"/>
+      <c r="K71" s="12" t="inlineStr"/>
+      <c r="L71" s="12" t="inlineStr"/>
+      <c r="M71" s="12" t="inlineStr"/>
+      <c r="N71" s="12" t="inlineStr"/>
+      <c r="O71" s="12" t="inlineStr"/>
+      <c r="P71" s="12" t="inlineStr"/>
+      <c r="Q71" s="12" t="inlineStr"/>
+      <c r="R71" s="12" t="inlineStr"/>
+      <c r="S71" s="12" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="inlineStr"/>
-      <c r="B72" s="5" t="inlineStr"/>
-      <c r="C72" s="5" t="inlineStr"/>
-      <c r="D72" s="5" t="inlineStr"/>
-      <c r="E72" s="5" t="inlineStr"/>
-      <c r="F72" s="5" t="inlineStr"/>
-      <c r="G72" s="5" t="inlineStr"/>
-      <c r="H72" s="5" t="inlineStr"/>
-      <c r="I72" s="5" t="inlineStr"/>
-      <c r="J72" s="5" t="inlineStr"/>
-      <c r="K72" s="5" t="inlineStr"/>
-      <c r="L72" s="5" t="inlineStr"/>
-      <c r="M72" s="5" t="inlineStr"/>
-      <c r="N72" s="5" t="inlineStr"/>
-      <c r="O72" s="5" t="inlineStr"/>
-      <c r="P72" s="5" t="inlineStr"/>
-      <c r="Q72" s="5" t="inlineStr"/>
-      <c r="R72" s="5" t="inlineStr"/>
-      <c r="S72" s="5" t="inlineStr"/>
+      <c r="A72" s="12" t="inlineStr"/>
+      <c r="B72" s="12" t="inlineStr"/>
+      <c r="C72" s="12" t="inlineStr"/>
+      <c r="D72" s="12" t="inlineStr"/>
+      <c r="E72" s="12" t="inlineStr"/>
+      <c r="F72" s="12" t="inlineStr"/>
+      <c r="G72" s="12" t="inlineStr"/>
+      <c r="H72" s="12" t="inlineStr"/>
+      <c r="I72" s="12" t="inlineStr"/>
+      <c r="J72" s="12" t="inlineStr"/>
+      <c r="K72" s="12" t="inlineStr"/>
+      <c r="L72" s="12" t="inlineStr"/>
+      <c r="M72" s="12" t="inlineStr"/>
+      <c r="N72" s="12" t="inlineStr"/>
+      <c r="O72" s="12" t="inlineStr"/>
+      <c r="P72" s="12" t="inlineStr"/>
+      <c r="Q72" s="12" t="inlineStr"/>
+      <c r="R72" s="12" t="inlineStr"/>
+      <c r="S72" s="12" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr"/>
-      <c r="B73" s="5" t="inlineStr"/>
-      <c r="C73" s="5" t="inlineStr"/>
-      <c r="D73" s="5" t="inlineStr"/>
-      <c r="E73" s="5" t="inlineStr"/>
-      <c r="F73" s="5" t="inlineStr"/>
-      <c r="G73" s="5" t="inlineStr"/>
-      <c r="H73" s="5" t="inlineStr"/>
-      <c r="I73" s="5" t="inlineStr"/>
-      <c r="J73" s="5" t="inlineStr"/>
-      <c r="K73" s="5" t="inlineStr"/>
-      <c r="L73" s="5" t="inlineStr"/>
-      <c r="M73" s="5" t="inlineStr"/>
-      <c r="N73" s="5" t="inlineStr"/>
-      <c r="O73" s="5" t="inlineStr"/>
-      <c r="P73" s="5" t="inlineStr"/>
-      <c r="Q73" s="5" t="inlineStr"/>
-      <c r="R73" s="5" t="inlineStr"/>
-      <c r="S73" s="5" t="inlineStr"/>
+      <c r="A73" s="12" t="inlineStr"/>
+      <c r="B73" s="12" t="inlineStr"/>
+      <c r="C73" s="12" t="inlineStr"/>
+      <c r="D73" s="12" t="inlineStr"/>
+      <c r="E73" s="12" t="inlineStr"/>
+      <c r="F73" s="12" t="inlineStr"/>
+      <c r="G73" s="12" t="inlineStr"/>
+      <c r="H73" s="12" t="inlineStr"/>
+      <c r="I73" s="12" t="inlineStr"/>
+      <c r="J73" s="12" t="inlineStr"/>
+      <c r="K73" s="12" t="inlineStr"/>
+      <c r="L73" s="12" t="inlineStr"/>
+      <c r="M73" s="12" t="inlineStr"/>
+      <c r="N73" s="12" t="inlineStr"/>
+      <c r="O73" s="12" t="inlineStr"/>
+      <c r="P73" s="12" t="inlineStr"/>
+      <c r="Q73" s="12" t="inlineStr"/>
+      <c r="R73" s="12" t="inlineStr"/>
+      <c r="S73" s="12" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="5" t="inlineStr"/>
-      <c r="B74" s="5" t="inlineStr"/>
-      <c r="C74" s="5" t="inlineStr"/>
-      <c r="D74" s="5" t="inlineStr"/>
-      <c r="E74" s="5" t="inlineStr"/>
-      <c r="F74" s="5" t="inlineStr"/>
-      <c r="G74" s="5" t="inlineStr"/>
-      <c r="H74" s="5" t="inlineStr"/>
-      <c r="I74" s="5" t="inlineStr"/>
-      <c r="J74" s="5" t="inlineStr"/>
-      <c r="K74" s="5" t="inlineStr"/>
-      <c r="L74" s="5" t="inlineStr"/>
-      <c r="M74" s="5" t="inlineStr"/>
-      <c r="N74" s="5" t="inlineStr"/>
-      <c r="O74" s="5" t="inlineStr"/>
-      <c r="P74" s="5" t="inlineStr"/>
-      <c r="Q74" s="5" t="inlineStr"/>
-      <c r="R74" s="5" t="inlineStr"/>
-      <c r="S74" s="5" t="inlineStr"/>
+      <c r="A74" s="12" t="inlineStr"/>
+      <c r="B74" s="12" t="inlineStr"/>
+      <c r="C74" s="12" t="inlineStr"/>
+      <c r="D74" s="12" t="inlineStr"/>
+      <c r="E74" s="12" t="inlineStr"/>
+      <c r="F74" s="12" t="inlineStr"/>
+      <c r="G74" s="12" t="inlineStr"/>
+      <c r="H74" s="12" t="inlineStr"/>
+      <c r="I74" s="12" t="inlineStr"/>
+      <c r="J74" s="12" t="inlineStr"/>
+      <c r="K74" s="12" t="inlineStr"/>
+      <c r="L74" s="12" t="inlineStr"/>
+      <c r="M74" s="12" t="inlineStr"/>
+      <c r="N74" s="12" t="inlineStr"/>
+      <c r="O74" s="12" t="inlineStr"/>
+      <c r="P74" s="12" t="inlineStr"/>
+      <c r="Q74" s="12" t="inlineStr"/>
+      <c r="R74" s="12" t="inlineStr"/>
+      <c r="S74" s="12" t="inlineStr"/>
     </row>
     <row r="75"/>
     <row r="76">
-      <c r="A76" s="7" t="inlineStr">
+      <c r="A76" s="14" t="inlineStr">
         <is>
           <t>增资配股</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+      <c r="A77" s="9" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="B77" s="9" t="inlineStr">
         <is>
           <t>认购人
 allottee_name</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="C77" s="9" t="inlineStr">
         <is>
           <t>认购人证件/注册号
 allottee_id_number</t>
         </is>
       </c>
-      <c r="D77" s="2" t="inlineStr">
+      <c r="D77" s="9" t="inlineStr">
         <is>
           <t>认购人地址
 allottee_address</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
+      <c r="E77" s="9" t="inlineStr">
         <is>
           <t>配发股数
 shares_allotted</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="F77" s="9" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="G77" s="2" t="inlineStr">
+      <c r="G77" s="9" t="inlineStr">
         <is>
           <t>本次已发行股本
 issued_share_capital</t>
         </is>
       </c>
-      <c r="H77" s="2" t="inlineStr">
+      <c r="H77" s="9" t="inlineStr">
         <is>
           <t>每股实缴
 amount_paid_per_share</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
+      <c r="I77" s="9" t="inlineStr">
         <is>
           <t>本次实缴资本
 total_paid</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr">
+      <c r="J77" s="9" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="K77" s="2" t="inlineStr">
+      <c r="K77" s="9" t="inlineStr">
         <is>
           <t>配股日期
 allotment_date</t>
         </is>
       </c>
-      <c r="L77" s="2" t="inlineStr">
+      <c r="L77" s="9" t="inlineStr">
         <is>
           <t>授权日期
 authority_date</t>
         </is>
       </c>
-      <c r="M77" s="2" t="inlineStr">
+      <c r="M77" s="9" t="inlineStr">
         <is>
           <t>是否 Form 24
 form24_required</t>
         </is>
       </c>
-      <c r="N77" s="2" t="inlineStr">
+      <c r="N77" s="9" t="inlineStr">
         <is>
           <t>证书号
 certificate_no</t>
         </is>
       </c>
-      <c r="O77" s="2" t="inlineStr">
+      <c r="O77" s="9" t="inlineStr">
         <is>
           <t>是否生成证书
 generate_certificate</t>
         </is>
       </c>
-      <c r="P77" s="2" t="inlineStr">
+      <c r="P77" s="9" t="inlineStr">
         <is>
           <t>配股后总股数
 post_allotment_total_shares</t>
         </is>
       </c>
-      <c r="Q77" s="2" t="inlineStr">
+      <c r="Q77" s="9" t="inlineStr">
         <is>
           <t>配股后已发行股本
 post_allotment_issued_share_capital</t>
         </is>
       </c>
-      <c r="R77" s="2" t="inlineStr">
+      <c r="R77" s="9" t="inlineStr">
         <is>
           <t>配股后实缴资本
 post_allotment_paid_up_capital</t>
         </is>
       </c>
-      <c r="S77" s="2" t="inlineStr">
+      <c r="S77" s="9" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -2218,178 +2247,178 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="5" t="inlineStr"/>
-      <c r="B78" s="5" t="inlineStr"/>
-      <c r="C78" s="5" t="inlineStr"/>
-      <c r="D78" s="5" t="inlineStr"/>
-      <c r="E78" s="5" t="inlineStr"/>
-      <c r="F78" s="5" t="inlineStr"/>
-      <c r="G78" s="5" t="inlineStr"/>
-      <c r="H78" s="5" t="inlineStr"/>
-      <c r="I78" s="5" t="inlineStr"/>
-      <c r="J78" s="5" t="inlineStr"/>
-      <c r="K78" s="5" t="inlineStr"/>
-      <c r="L78" s="5" t="inlineStr"/>
-      <c r="M78" s="5" t="inlineStr"/>
-      <c r="N78" s="5" t="inlineStr"/>
-      <c r="O78" s="5" t="inlineStr"/>
-      <c r="P78" s="5" t="inlineStr"/>
-      <c r="Q78" s="5" t="inlineStr"/>
-      <c r="R78" s="5" t="inlineStr"/>
-      <c r="S78" s="5" t="inlineStr"/>
+      <c r="A78" s="12" t="inlineStr"/>
+      <c r="B78" s="12" t="inlineStr"/>
+      <c r="C78" s="12" t="inlineStr"/>
+      <c r="D78" s="12" t="inlineStr"/>
+      <c r="E78" s="12" t="inlineStr"/>
+      <c r="F78" s="12" t="inlineStr"/>
+      <c r="G78" s="12" t="inlineStr"/>
+      <c r="H78" s="12" t="inlineStr"/>
+      <c r="I78" s="12" t="inlineStr"/>
+      <c r="J78" s="12" t="inlineStr"/>
+      <c r="K78" s="12" t="inlineStr"/>
+      <c r="L78" s="12" t="inlineStr"/>
+      <c r="M78" s="12" t="inlineStr"/>
+      <c r="N78" s="12" t="inlineStr"/>
+      <c r="O78" s="12" t="inlineStr"/>
+      <c r="P78" s="12" t="inlineStr"/>
+      <c r="Q78" s="12" t="inlineStr"/>
+      <c r="R78" s="12" t="inlineStr"/>
+      <c r="S78" s="12" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="5" t="inlineStr"/>
-      <c r="B79" s="5" t="inlineStr"/>
-      <c r="C79" s="5" t="inlineStr"/>
-      <c r="D79" s="5" t="inlineStr"/>
-      <c r="E79" s="5" t="inlineStr"/>
-      <c r="F79" s="5" t="inlineStr"/>
-      <c r="G79" s="5" t="inlineStr"/>
-      <c r="H79" s="5" t="inlineStr"/>
-      <c r="I79" s="5" t="inlineStr"/>
-      <c r="J79" s="5" t="inlineStr"/>
-      <c r="K79" s="5" t="inlineStr"/>
-      <c r="L79" s="5" t="inlineStr"/>
-      <c r="M79" s="5" t="inlineStr"/>
-      <c r="N79" s="5" t="inlineStr"/>
-      <c r="O79" s="5" t="inlineStr"/>
-      <c r="P79" s="5" t="inlineStr"/>
-      <c r="Q79" s="5" t="inlineStr"/>
-      <c r="R79" s="5" t="inlineStr"/>
-      <c r="S79" s="5" t="inlineStr"/>
+      <c r="A79" s="12" t="inlineStr"/>
+      <c r="B79" s="12" t="inlineStr"/>
+      <c r="C79" s="12" t="inlineStr"/>
+      <c r="D79" s="12" t="inlineStr"/>
+      <c r="E79" s="12" t="inlineStr"/>
+      <c r="F79" s="12" t="inlineStr"/>
+      <c r="G79" s="12" t="inlineStr"/>
+      <c r="H79" s="12" t="inlineStr"/>
+      <c r="I79" s="12" t="inlineStr"/>
+      <c r="J79" s="12" t="inlineStr"/>
+      <c r="K79" s="12" t="inlineStr"/>
+      <c r="L79" s="12" t="inlineStr"/>
+      <c r="M79" s="12" t="inlineStr"/>
+      <c r="N79" s="12" t="inlineStr"/>
+      <c r="O79" s="12" t="inlineStr"/>
+      <c r="P79" s="12" t="inlineStr"/>
+      <c r="Q79" s="12" t="inlineStr"/>
+      <c r="R79" s="12" t="inlineStr"/>
+      <c r="S79" s="12" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="5" t="inlineStr"/>
-      <c r="B80" s="5" t="inlineStr"/>
-      <c r="C80" s="5" t="inlineStr"/>
-      <c r="D80" s="5" t="inlineStr"/>
-      <c r="E80" s="5" t="inlineStr"/>
-      <c r="F80" s="5" t="inlineStr"/>
-      <c r="G80" s="5" t="inlineStr"/>
-      <c r="H80" s="5" t="inlineStr"/>
-      <c r="I80" s="5" t="inlineStr"/>
-      <c r="J80" s="5" t="inlineStr"/>
-      <c r="K80" s="5" t="inlineStr"/>
-      <c r="L80" s="5" t="inlineStr"/>
-      <c r="M80" s="5" t="inlineStr"/>
-      <c r="N80" s="5" t="inlineStr"/>
-      <c r="O80" s="5" t="inlineStr"/>
-      <c r="P80" s="5" t="inlineStr"/>
-      <c r="Q80" s="5" t="inlineStr"/>
-      <c r="R80" s="5" t="inlineStr"/>
-      <c r="S80" s="5" t="inlineStr"/>
+      <c r="A80" s="12" t="inlineStr"/>
+      <c r="B80" s="12" t="inlineStr"/>
+      <c r="C80" s="12" t="inlineStr"/>
+      <c r="D80" s="12" t="inlineStr"/>
+      <c r="E80" s="12" t="inlineStr"/>
+      <c r="F80" s="12" t="inlineStr"/>
+      <c r="G80" s="12" t="inlineStr"/>
+      <c r="H80" s="12" t="inlineStr"/>
+      <c r="I80" s="12" t="inlineStr"/>
+      <c r="J80" s="12" t="inlineStr"/>
+      <c r="K80" s="12" t="inlineStr"/>
+      <c r="L80" s="12" t="inlineStr"/>
+      <c r="M80" s="12" t="inlineStr"/>
+      <c r="N80" s="12" t="inlineStr"/>
+      <c r="O80" s="12" t="inlineStr"/>
+      <c r="P80" s="12" t="inlineStr"/>
+      <c r="Q80" s="12" t="inlineStr"/>
+      <c r="R80" s="12" t="inlineStr"/>
+      <c r="S80" s="12" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="inlineStr"/>
-      <c r="B81" s="5" t="inlineStr"/>
-      <c r="C81" s="5" t="inlineStr"/>
-      <c r="D81" s="5" t="inlineStr"/>
-      <c r="E81" s="5" t="inlineStr"/>
-      <c r="F81" s="5" t="inlineStr"/>
-      <c r="G81" s="5" t="inlineStr"/>
-      <c r="H81" s="5" t="inlineStr"/>
-      <c r="I81" s="5" t="inlineStr"/>
-      <c r="J81" s="5" t="inlineStr"/>
-      <c r="K81" s="5" t="inlineStr"/>
-      <c r="L81" s="5" t="inlineStr"/>
-      <c r="M81" s="5" t="inlineStr"/>
-      <c r="N81" s="5" t="inlineStr"/>
-      <c r="O81" s="5" t="inlineStr"/>
-      <c r="P81" s="5" t="inlineStr"/>
-      <c r="Q81" s="5" t="inlineStr"/>
-      <c r="R81" s="5" t="inlineStr"/>
-      <c r="S81" s="5" t="inlineStr"/>
+      <c r="A81" s="12" t="inlineStr"/>
+      <c r="B81" s="12" t="inlineStr"/>
+      <c r="C81" s="12" t="inlineStr"/>
+      <c r="D81" s="12" t="inlineStr"/>
+      <c r="E81" s="12" t="inlineStr"/>
+      <c r="F81" s="12" t="inlineStr"/>
+      <c r="G81" s="12" t="inlineStr"/>
+      <c r="H81" s="12" t="inlineStr"/>
+      <c r="I81" s="12" t="inlineStr"/>
+      <c r="J81" s="12" t="inlineStr"/>
+      <c r="K81" s="12" t="inlineStr"/>
+      <c r="L81" s="12" t="inlineStr"/>
+      <c r="M81" s="12" t="inlineStr"/>
+      <c r="N81" s="12" t="inlineStr"/>
+      <c r="O81" s="12" t="inlineStr"/>
+      <c r="P81" s="12" t="inlineStr"/>
+      <c r="Q81" s="12" t="inlineStr"/>
+      <c r="R81" s="12" t="inlineStr"/>
+      <c r="S81" s="12" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="inlineStr"/>
-      <c r="B82" s="5" t="inlineStr"/>
-      <c r="C82" s="5" t="inlineStr"/>
-      <c r="D82" s="5" t="inlineStr"/>
-      <c r="E82" s="5" t="inlineStr"/>
-      <c r="F82" s="5" t="inlineStr"/>
-      <c r="G82" s="5" t="inlineStr"/>
-      <c r="H82" s="5" t="inlineStr"/>
-      <c r="I82" s="5" t="inlineStr"/>
-      <c r="J82" s="5" t="inlineStr"/>
-      <c r="K82" s="5" t="inlineStr"/>
-      <c r="L82" s="5" t="inlineStr"/>
-      <c r="M82" s="5" t="inlineStr"/>
-      <c r="N82" s="5" t="inlineStr"/>
-      <c r="O82" s="5" t="inlineStr"/>
-      <c r="P82" s="5" t="inlineStr"/>
-      <c r="Q82" s="5" t="inlineStr"/>
-      <c r="R82" s="5" t="inlineStr"/>
-      <c r="S82" s="5" t="inlineStr"/>
+      <c r="A82" s="12" t="inlineStr"/>
+      <c r="B82" s="12" t="inlineStr"/>
+      <c r="C82" s="12" t="inlineStr"/>
+      <c r="D82" s="12" t="inlineStr"/>
+      <c r="E82" s="12" t="inlineStr"/>
+      <c r="F82" s="12" t="inlineStr"/>
+      <c r="G82" s="12" t="inlineStr"/>
+      <c r="H82" s="12" t="inlineStr"/>
+      <c r="I82" s="12" t="inlineStr"/>
+      <c r="J82" s="12" t="inlineStr"/>
+      <c r="K82" s="12" t="inlineStr"/>
+      <c r="L82" s="12" t="inlineStr"/>
+      <c r="M82" s="12" t="inlineStr"/>
+      <c r="N82" s="12" t="inlineStr"/>
+      <c r="O82" s="12" t="inlineStr"/>
+      <c r="P82" s="12" t="inlineStr"/>
+      <c r="Q82" s="12" t="inlineStr"/>
+      <c r="R82" s="12" t="inlineStr"/>
+      <c r="S82" s="12" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="5" t="inlineStr"/>
-      <c r="B83" s="5" t="inlineStr"/>
-      <c r="C83" s="5" t="inlineStr"/>
-      <c r="D83" s="5" t="inlineStr"/>
-      <c r="E83" s="5" t="inlineStr"/>
-      <c r="F83" s="5" t="inlineStr"/>
-      <c r="G83" s="5" t="inlineStr"/>
-      <c r="H83" s="5" t="inlineStr"/>
-      <c r="I83" s="5" t="inlineStr"/>
-      <c r="J83" s="5" t="inlineStr"/>
-      <c r="K83" s="5" t="inlineStr"/>
-      <c r="L83" s="5" t="inlineStr"/>
-      <c r="M83" s="5" t="inlineStr"/>
-      <c r="N83" s="5" t="inlineStr"/>
-      <c r="O83" s="5" t="inlineStr"/>
-      <c r="P83" s="5" t="inlineStr"/>
-      <c r="Q83" s="5" t="inlineStr"/>
-      <c r="R83" s="5" t="inlineStr"/>
-      <c r="S83" s="5" t="inlineStr"/>
+      <c r="A83" s="12" t="inlineStr"/>
+      <c r="B83" s="12" t="inlineStr"/>
+      <c r="C83" s="12" t="inlineStr"/>
+      <c r="D83" s="12" t="inlineStr"/>
+      <c r="E83" s="12" t="inlineStr"/>
+      <c r="F83" s="12" t="inlineStr"/>
+      <c r="G83" s="12" t="inlineStr"/>
+      <c r="H83" s="12" t="inlineStr"/>
+      <c r="I83" s="12" t="inlineStr"/>
+      <c r="J83" s="12" t="inlineStr"/>
+      <c r="K83" s="12" t="inlineStr"/>
+      <c r="L83" s="12" t="inlineStr"/>
+      <c r="M83" s="12" t="inlineStr"/>
+      <c r="N83" s="12" t="inlineStr"/>
+      <c r="O83" s="12" t="inlineStr"/>
+      <c r="P83" s="12" t="inlineStr"/>
+      <c r="Q83" s="12" t="inlineStr"/>
+      <c r="R83" s="12" t="inlineStr"/>
+      <c r="S83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="5" t="inlineStr"/>
-      <c r="B84" s="5" t="inlineStr"/>
-      <c r="C84" s="5" t="inlineStr"/>
-      <c r="D84" s="5" t="inlineStr"/>
-      <c r="E84" s="5" t="inlineStr"/>
-      <c r="F84" s="5" t="inlineStr"/>
-      <c r="G84" s="5" t="inlineStr"/>
-      <c r="H84" s="5" t="inlineStr"/>
-      <c r="I84" s="5" t="inlineStr"/>
-      <c r="J84" s="5" t="inlineStr"/>
-      <c r="K84" s="5" t="inlineStr"/>
-      <c r="L84" s="5" t="inlineStr"/>
-      <c r="M84" s="5" t="inlineStr"/>
-      <c r="N84" s="5" t="inlineStr"/>
-      <c r="O84" s="5" t="inlineStr"/>
-      <c r="P84" s="5" t="inlineStr"/>
-      <c r="Q84" s="5" t="inlineStr"/>
-      <c r="R84" s="5" t="inlineStr"/>
-      <c r="S84" s="5" t="inlineStr"/>
+      <c r="A84" s="12" t="inlineStr"/>
+      <c r="B84" s="12" t="inlineStr"/>
+      <c r="C84" s="12" t="inlineStr"/>
+      <c r="D84" s="12" t="inlineStr"/>
+      <c r="E84" s="12" t="inlineStr"/>
+      <c r="F84" s="12" t="inlineStr"/>
+      <c r="G84" s="12" t="inlineStr"/>
+      <c r="H84" s="12" t="inlineStr"/>
+      <c r="I84" s="12" t="inlineStr"/>
+      <c r="J84" s="12" t="inlineStr"/>
+      <c r="K84" s="12" t="inlineStr"/>
+      <c r="L84" s="12" t="inlineStr"/>
+      <c r="M84" s="12" t="inlineStr"/>
+      <c r="N84" s="12" t="inlineStr"/>
+      <c r="O84" s="12" t="inlineStr"/>
+      <c r="P84" s="12" t="inlineStr"/>
+      <c r="Q84" s="12" t="inlineStr"/>
+      <c r="R84" s="12" t="inlineStr"/>
+      <c r="S84" s="12" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="5" t="inlineStr"/>
-      <c r="B85" s="5" t="inlineStr"/>
-      <c r="C85" s="5" t="inlineStr"/>
-      <c r="D85" s="5" t="inlineStr"/>
-      <c r="E85" s="5" t="inlineStr"/>
-      <c r="F85" s="5" t="inlineStr"/>
-      <c r="G85" s="5" t="inlineStr"/>
-      <c r="H85" s="5" t="inlineStr"/>
-      <c r="I85" s="5" t="inlineStr"/>
-      <c r="J85" s="5" t="inlineStr"/>
-      <c r="K85" s="5" t="inlineStr"/>
-      <c r="L85" s="5" t="inlineStr"/>
-      <c r="M85" s="5" t="inlineStr"/>
-      <c r="N85" s="5" t="inlineStr"/>
-      <c r="O85" s="5" t="inlineStr"/>
-      <c r="P85" s="5" t="inlineStr"/>
-      <c r="Q85" s="5" t="inlineStr"/>
-      <c r="R85" s="5" t="inlineStr"/>
-      <c r="S85" s="5" t="inlineStr"/>
+      <c r="A85" s="12" t="inlineStr"/>
+      <c r="B85" s="12" t="inlineStr"/>
+      <c r="C85" s="12" t="inlineStr"/>
+      <c r="D85" s="12" t="inlineStr"/>
+      <c r="E85" s="12" t="inlineStr"/>
+      <c r="F85" s="12" t="inlineStr"/>
+      <c r="G85" s="12" t="inlineStr"/>
+      <c r="H85" s="12" t="inlineStr"/>
+      <c r="I85" s="12" t="inlineStr"/>
+      <c r="J85" s="12" t="inlineStr"/>
+      <c r="K85" s="12" t="inlineStr"/>
+      <c r="L85" s="12" t="inlineStr"/>
+      <c r="M85" s="12" t="inlineStr"/>
+      <c r="N85" s="12" t="inlineStr"/>
+      <c r="O85" s="12" t="inlineStr"/>
+      <c r="P85" s="12" t="inlineStr"/>
+      <c r="Q85" s="12" t="inlineStr"/>
+      <c r="R85" s="12" t="inlineStr"/>
+      <c r="S85" s="12" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="19">
+  <dataValidations count="18">
     <dataValidation sqref="D19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
@@ -2401,9 +2430,6 @@
     </dataValidation>
     <dataValidation sqref="D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation sqref="D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"cooperative,non_cooperative"</formula1>
     </dataValidation>
     <dataValidation sqref="D35" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
@@ -2470,7 +2496,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>快速年审 Annual Review - 常用默认值已内置</t>
         </is>
@@ -2478,764 +2504,764 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>field_key</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t>填写内容 / Value</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>是否做年审</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Annual review required</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>annual_review_required</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D4" s="12" t="inlineStr"/>
+      <c r="E4" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>财年结束日</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>Financial year end</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>fye_date</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="D5" s="12" t="inlineStr"/>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>AGM 日期</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="10" t="inlineStr">
         <is>
           <t>AGM date</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>agm_date</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="D6" s="12" t="inlineStr"/>
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>建议填</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>留空后续可由系统按规则推定。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>AGM 时间</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>AGM time</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>agm_time</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>10.00 a.m.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>通常不用改。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>AGM 地点</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>AGM place</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>agm_place</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr"/>
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>默认注册地址</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>留空默认当前注册地址。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>年审方式</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>AGM route</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>agm_route</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>ordinary_agm</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>ordinary_agm / exempt_private_company / dormant_company / manual。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>财报状态</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Accounts status</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>accounts_status</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>non_dormant</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>常用</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>non_dormant / dormant / unaudited / audited。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="10" t="inlineStr">
         <is>
           <t>公司活动状态</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="10" t="inlineStr">
         <is>
           <t>Company activity status</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>company_activity_status</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Active / Dormant；留空按 Active。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>是否 ACRA 休眠相关公司</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>ACRA dormant relevant company</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>acra_dormant_relevant_company</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F12" s="6" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Auto / Yes / No；休眠公司会影响是否需要财报。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>资产是否不超过 50 万</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" s="10" t="inlineStr">
         <is>
           <t>Total assets under S$500k</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>total_assets_under_500k</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Auto / Yes / No；用于判断 dormant AGM exemption 风险。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>是否需要财报</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" s="10" t="inlineStr">
         <is>
           <t>Financial statements required</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>financial_statements_required</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Auto / Yes / No；休眠且符合条件时可 No。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>财报类型</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Financial statements type</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>financial_statements_type</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Auto / Unaudited / Audited / Dormant no FS / Management accounts。</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>审计/豁免状态</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>Audit exemption status</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>audit_exemption_status</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Auto / Small company exempt / Audited / Dormant relevant / Manual review。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>AGM 状态</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>AGM status</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>agm_status</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Auto / Held AGM / Dispensed with AGM / Exempt from AGM / Written resolutions。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>IRAS 税务状态</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>IRAS tax status</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>iras_tax_status</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Auto / Active / Dormant / Dormant waiver granted / Manual review；只作复核提醒。</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>财报日期</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>Financial statement date</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>financial_statement_date</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr"/>
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>默认 FYE</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>留空默认财年结束日。</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>董事签字人</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" s="10" t="inlineStr">
         <is>
           <t>Director signer</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>director_signer_name</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D20" s="12" t="inlineStr"/>
+      <c r="E20" s="10" t="inlineStr">
         <is>
           <t>常用</t>
         </is>
       </c>
-      <c r="F20" s="6" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>留空默认首页董事签字人。</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>股东/成员签字人</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>Shareholder signer</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>shareholder_signer_name</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D21" s="12" t="inlineStr"/>
+      <c r="E21" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>需要股东签署的年审文件使用。</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>AR 授权签字人</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>AR authorised signer</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>ar_authorized_signer_name</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr"/>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="D22" s="12" t="inlineStr"/>
+      <c r="E22" s="10" t="inlineStr">
         <is>
           <t>默认董事签字人</t>
         </is>
       </c>
-      <c r="F22" s="6" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Annual Return 授权。</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>董事费</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="10" t="inlineStr">
         <is>
           <t>Directors' fee</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>directors_fee</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>通常 0。</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>董事薪酬</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>Directors' remuneration</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>directors_remuneration</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F24" s="6" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>通常 0。</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Shorter Notice Consent</t>
         </is>
       </c>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" s="10" t="inlineStr">
         <is>
           <t>Shorter notice consent</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>shorter_notice_consent</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="12" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>Auto / Yes / No。</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Management Representation Letter</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>MRL</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>management_rep_letter</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D26" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="10" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F26" s="6" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>Yes / No。</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" s="10" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr"/>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="D27" s="12" t="inlineStr"/>
+      <c r="E27" s="10" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>特殊情况写这里。</t>
         </is>

</xml_diff>

<commit_message>
Improve annual review output and field highlighting
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -110,27 +110,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -540,7 +521,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>P2 一页式快速业务单 - 少填字段先生成文件</t>
         </is>
@@ -548,1048 +529,1048 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>field_key</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>填写内容 / Value</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>公司名称</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Company name</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>所有文件都会用。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>UEN / 注册号</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>UEN</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>uen</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>现有公司变更建议填写。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>当前注册地址</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Current registered office</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>registered_office_address</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>多数文件会用；地址变更时作为旧地址。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>当前总股数</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Current total shares</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>total_issued_shares</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr"/>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>用于增资配股后资本推导；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>当前已发行股本</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Current issued share capital</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>issued_share_capital</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>对应 ACRA issued share capital；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>当前实缴资本</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Current paid-up share capital</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>paid_up_capital</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr"/>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>M04 可空</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>对应 ACRA paid-up share capital；不知道可留空。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>币种</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>SGD</t>
         </is>
       </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>通常 SGD；如 USD 等请填写。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>文件日期</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Document date</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>default_document_date</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr"/>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>建议必填</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY；留空后续可由网页补当天。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>M01 directors to sign</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>M01 director signer names</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>director_signer_names</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr"/>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Recommended</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Enter all current directors for M01. One per line, comma, or semicolon.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>股东/成员签字人姓名</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Member/shareholder signer names</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>member_signer_names</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr"/>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>转入建议填</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>M02 股东/成员签署处使用；多人可换行、逗号或分号分隔。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>客户方签字人姓名</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Client signer name</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>client_signatory_name</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr"/>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>交接信签字人；留空默认用第一个股东/成员签字人。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>业务单编号</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Business order ID</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>business_order_id</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr"/>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>后台预留。</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>数据来源</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Source type</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>source_type</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>AI / BizFile / Excel / Manual。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>来源文件编号</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Source file ID</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>source_file_id</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr"/>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>可填 BizFile 或旧表文件名。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>经办人</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Prepared by</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>prepared_by</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr"/>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>内部记录。</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>是否变更注册地址</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Change registered office</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>change_registered_office_required</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr"/>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新注册地址即可生成；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>新注册地址</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>New registered office</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>new_registered_office_address</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>地址变更时填</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr"/>
+      <c r="F20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>是否变更营业范围</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Change business activity</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>change_business_activity_required</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新 SSIC/业务范围即可生成；填 No 则不生成。支持主业务和副业务。</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>新主 SSIC</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>New primary SSIC</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>new_primary_ssic</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr"/>
+      <c r="F22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>新主营业范围</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>New primary activity</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>new_primary_activity</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr"/>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>营业范围变更时填</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr"/>
+      <c r="F23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>新副 SSIC</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>New secondary SSIC</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>new_secondary_ssic</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr"/>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr"/>
+      <c r="F24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>新副营业范围</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>New secondary activity</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>new_secondary_activity</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr"/>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr"/>
+      <c r="F25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>是否变更 FYE</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Change FYE</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>change_fye_required</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr"/>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写新 FYE 即可生成；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>旧 FYE</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Old FYE</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>old_fye</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr"/>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>FYE 变更时填</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>新 FYE</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>New FYE</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>new_fye</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr"/>
-      <c r="E28" s="10" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>FYE 变更时填</t>
         </is>
       </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="F28" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>下个账期开始</t>
         </is>
       </c>
-      <c r="B29" s="10" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Next accounts period start</t>
         </is>
       </c>
-      <c r="C29" s="11" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>next_accounts_period_start</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr"/>
-      <c r="E29" s="10" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F29" s="13" t="inlineStr"/>
+      <c r="F29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>下个账期结束</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>Next accounts period end</t>
         </is>
       </c>
-      <c r="C30" s="11" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>next_accounts_period_end</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr"/>
-      <c r="E30" s="10" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F30" s="13" t="inlineStr"/>
+      <c r="F30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>是否转入秘书公司</t>
         </is>
       </c>
-      <c r="B31" s="10" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
         <is>
           <t>Transfer-in required</t>
         </is>
       </c>
-      <c r="C31" s="11" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>transfer_in_required</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr"/>
-      <c r="E31" s="10" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>需要时填 Yes</t>
         </is>
       </c>
-      <c r="F31" s="13" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
         <is>
           <t>转入需要时填 Yes；M01 正常出，M02 一律兜底。</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>转入模式</t>
         </is>
       </c>
-      <c r="B32" s="10" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Transfer-in mode</t>
         </is>
       </c>
-      <c r="C32" s="11" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>transfer_in_mode</t>
         </is>
       </c>
-      <c r="D32" s="12" t="inlineStr"/>
-      <c r="E32" s="10" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>内部预留</t>
         </is>
       </c>
-      <c r="F32" s="13" t="inlineStr">
+      <c r="F32" s="6" t="inlineStr">
         <is>
           <t>通常留空；系统不再要求区分配合/不配合。</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="10" t="inlineStr">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>旧秘书公司</t>
         </is>
       </c>
-      <c r="B33" s="10" t="inlineStr">
+      <c r="B33" s="3" t="inlineStr">
         <is>
           <t>Old secretary firm</t>
         </is>
       </c>
-      <c r="C33" s="11" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>old_secretary_company</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr"/>
-      <c r="E33" s="10" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F33" s="13" t="inlineStr"/>
+      <c r="F33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="10" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>新秘书公司</t>
         </is>
       </c>
-      <c r="B34" s="10" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>New secretary firm</t>
         </is>
       </c>
-      <c r="C34" s="11" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>new_secretary_company</t>
         </is>
       </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>RSIN GROUP PTE. LTD.</t>
         </is>
       </c>
-      <c r="E34" s="10" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F34" s="13" t="inlineStr"/>
+      <c r="F34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>是否出辞职信</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>Generate resignation letter</t>
         </is>
       </c>
-      <c r="C35" s="11" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>generate_resignation_letter</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E35" s="10" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
         <is>
           <t>只有需要旧人员单独签辞职信时填 Yes；一般留 No。</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="10" t="inlineStr">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>是否做年审</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Annual review required</t>
         </is>
       </c>
-      <c r="C36" s="11" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>annual_review_required</t>
         </is>
       </c>
-      <c r="D36" s="12" t="inlineStr"/>
-      <c r="E36" s="10" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="F36" s="6" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>年审 FYE</t>
         </is>
       </c>
-      <c r="B37" s="10" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Annual review FYE</t>
         </is>
       </c>
-      <c r="C37" s="11" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>fye_date</t>
         </is>
       </c>
-      <c r="D37" s="12" t="inlineStr"/>
-      <c r="E37" s="10" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>年审时填</t>
         </is>
       </c>
-      <c r="F37" s="13" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="10" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>AGM 日期</t>
         </is>
       </c>
-      <c r="B38" s="10" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>AGM date</t>
         </is>
       </c>
-      <c r="C38" s="11" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>agm_date</t>
         </is>
       </c>
-      <c r="D38" s="12" t="inlineStr"/>
-      <c r="E38" s="10" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F38" s="13" t="inlineStr">
+      <c r="F38" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="10" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>年审备注</t>
         </is>
       </c>
-      <c r="B39" s="10" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
         <is>
           <t>Annual review remarks</t>
         </is>
       </c>
-      <c r="C39" s="11" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>annual_review_remarks</t>
         </is>
       </c>
-      <c r="D39" s="12" t="inlineStr"/>
-      <c r="E39" s="10" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F39" s="13" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
         <is>
           <t>复杂情况写这里；详细字段可填“快速年审”页。</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="10" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="B40" s="10" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="C40" s="11" t="inlineStr">
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="D40" s="12" t="inlineStr"/>
-      <c r="E40" s="10" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F40" s="13" t="inlineStr">
+      <c r="F40" s="6" t="inlineStr">
         <is>
           <t>内部备注，不进正式文件。</t>
         </is>
@@ -1598,44 +1579,44 @@
     <row r="41"/>
     <row r="42"/>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>人员任免</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="9" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B44" s="9" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>动作
 action_type</t>
         </is>
       </c>
-      <c r="C44" s="9" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="D44" s="9" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>是否出辞职信
 resignation_letter</t>
         </is>
       </c>
-      <c r="F44" s="9" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1643,115 +1624,115 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="12" t="inlineStr"/>
-      <c r="B45" s="12" t="inlineStr"/>
-      <c r="C45" s="12" t="inlineStr"/>
-      <c r="D45" s="12" t="inlineStr"/>
-      <c r="E45" s="12" t="inlineStr"/>
-      <c r="F45" s="12" t="inlineStr"/>
+      <c r="A45" s="5" t="inlineStr"/>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="12" t="inlineStr"/>
-      <c r="B46" s="12" t="inlineStr"/>
-      <c r="C46" s="12" t="inlineStr"/>
-      <c r="D46" s="12" t="inlineStr"/>
-      <c r="E46" s="12" t="inlineStr"/>
-      <c r="F46" s="12" t="inlineStr"/>
+      <c r="A46" s="5" t="inlineStr"/>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="inlineStr"/>
-      <c r="B47" s="12" t="inlineStr"/>
-      <c r="C47" s="12" t="inlineStr"/>
-      <c r="D47" s="12" t="inlineStr"/>
-      <c r="E47" s="12" t="inlineStr"/>
-      <c r="F47" s="12" t="inlineStr"/>
+      <c r="A47" s="5" t="inlineStr"/>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="12" t="inlineStr"/>
-      <c r="B48" s="12" t="inlineStr"/>
-      <c r="C48" s="12" t="inlineStr"/>
-      <c r="D48" s="12" t="inlineStr"/>
-      <c r="E48" s="12" t="inlineStr"/>
-      <c r="F48" s="12" t="inlineStr"/>
+      <c r="A48" s="5" t="inlineStr"/>
+      <c r="B48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="inlineStr"/>
-      <c r="B49" s="12" t="inlineStr"/>
-      <c r="C49" s="12" t="inlineStr"/>
-      <c r="D49" s="12" t="inlineStr"/>
-      <c r="E49" s="12" t="inlineStr"/>
-      <c r="F49" s="12" t="inlineStr"/>
+      <c r="A49" s="5" t="inlineStr"/>
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="inlineStr"/>
-      <c r="B50" s="12" t="inlineStr"/>
-      <c r="C50" s="12" t="inlineStr"/>
-      <c r="D50" s="12" t="inlineStr"/>
-      <c r="E50" s="12" t="inlineStr"/>
-      <c r="F50" s="12" t="inlineStr"/>
+      <c r="A50" s="5" t="inlineStr"/>
+      <c r="B50" s="5" t="inlineStr"/>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="5" t="inlineStr"/>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="inlineStr"/>
-      <c r="B51" s="12" t="inlineStr"/>
-      <c r="C51" s="12" t="inlineStr"/>
-      <c r="D51" s="12" t="inlineStr"/>
-      <c r="E51" s="12" t="inlineStr"/>
-      <c r="F51" s="12" t="inlineStr"/>
+      <c r="A51" s="5" t="inlineStr"/>
+      <c r="B51" s="5" t="inlineStr"/>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="5" t="inlineStr"/>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="12" t="inlineStr"/>
-      <c r="B52" s="12" t="inlineStr"/>
-      <c r="C52" s="12" t="inlineStr"/>
-      <c r="D52" s="12" t="inlineStr"/>
-      <c r="E52" s="12" t="inlineStr"/>
-      <c r="F52" s="12" t="inlineStr"/>
+      <c r="A52" s="5" t="inlineStr"/>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="5" t="inlineStr"/>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="inlineStr"/>
     </row>
     <row r="53"/>
     <row r="54">
-      <c r="A54" s="14" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>个人资料变更</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="9" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B55" s="9" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>变更字段
 field_label</t>
         </is>
       </c>
-      <c r="D55" s="9" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>原资料
 old_value</t>
         </is>
       </c>
-      <c r="E55" s="9" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>新资料
 new_value</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="2" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1759,195 +1740,195 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="inlineStr"/>
-      <c r="B56" s="12" t="inlineStr"/>
-      <c r="C56" s="12" t="inlineStr"/>
-      <c r="D56" s="12" t="inlineStr"/>
-      <c r="E56" s="12" t="inlineStr"/>
-      <c r="F56" s="12" t="inlineStr"/>
-      <c r="G56" s="12" t="inlineStr"/>
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="5" t="inlineStr"/>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="12" t="inlineStr"/>
-      <c r="B57" s="12" t="inlineStr"/>
-      <c r="C57" s="12" t="inlineStr"/>
-      <c r="D57" s="12" t="inlineStr"/>
-      <c r="E57" s="12" t="inlineStr"/>
-      <c r="F57" s="12" t="inlineStr"/>
-      <c r="G57" s="12" t="inlineStr"/>
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="inlineStr"/>
-      <c r="B58" s="12" t="inlineStr"/>
-      <c r="C58" s="12" t="inlineStr"/>
-      <c r="D58" s="12" t="inlineStr"/>
-      <c r="E58" s="12" t="inlineStr"/>
-      <c r="F58" s="12" t="inlineStr"/>
-      <c r="G58" s="12" t="inlineStr"/>
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr"/>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="12" t="inlineStr"/>
-      <c r="B59" s="12" t="inlineStr"/>
-      <c r="C59" s="12" t="inlineStr"/>
-      <c r="D59" s="12" t="inlineStr"/>
-      <c r="E59" s="12" t="inlineStr"/>
-      <c r="F59" s="12" t="inlineStr"/>
-      <c r="G59" s="12" t="inlineStr"/>
+      <c r="A59" s="5" t="inlineStr"/>
+      <c r="B59" s="5" t="inlineStr"/>
+      <c r="C59" s="5" t="inlineStr"/>
+      <c r="D59" s="5" t="inlineStr"/>
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="5" t="inlineStr"/>
+      <c r="G59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="12" t="inlineStr"/>
-      <c r="B60" s="12" t="inlineStr"/>
-      <c r="C60" s="12" t="inlineStr"/>
-      <c r="D60" s="12" t="inlineStr"/>
-      <c r="E60" s="12" t="inlineStr"/>
-      <c r="F60" s="12" t="inlineStr"/>
-      <c r="G60" s="12" t="inlineStr"/>
+      <c r="A60" s="5" t="inlineStr"/>
+      <c r="B60" s="5" t="inlineStr"/>
+      <c r="C60" s="5" t="inlineStr"/>
+      <c r="D60" s="5" t="inlineStr"/>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="12" t="inlineStr"/>
-      <c r="B61" s="12" t="inlineStr"/>
-      <c r="C61" s="12" t="inlineStr"/>
-      <c r="D61" s="12" t="inlineStr"/>
-      <c r="E61" s="12" t="inlineStr"/>
-      <c r="F61" s="12" t="inlineStr"/>
-      <c r="G61" s="12" t="inlineStr"/>
+      <c r="A61" s="5" t="inlineStr"/>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr"/>
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="12" t="inlineStr"/>
-      <c r="B62" s="12" t="inlineStr"/>
-      <c r="C62" s="12" t="inlineStr"/>
-      <c r="D62" s="12" t="inlineStr"/>
-      <c r="E62" s="12" t="inlineStr"/>
-      <c r="F62" s="12" t="inlineStr"/>
-      <c r="G62" s="12" t="inlineStr"/>
+      <c r="A62" s="5" t="inlineStr"/>
+      <c r="B62" s="5" t="inlineStr"/>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" s="12" t="inlineStr"/>
-      <c r="B63" s="12" t="inlineStr"/>
-      <c r="C63" s="12" t="inlineStr"/>
-      <c r="D63" s="12" t="inlineStr"/>
-      <c r="E63" s="12" t="inlineStr"/>
-      <c r="F63" s="12" t="inlineStr"/>
-      <c r="G63" s="12" t="inlineStr"/>
+      <c r="A63" s="5" t="inlineStr"/>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr"/>
     </row>
     <row r="64"/>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>股份转让</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="9" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B66" s="9" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>转让人
 transferor_name</t>
         </is>
       </c>
-      <c r="C66" s="9" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>转让人证件/注册号
 transferor_id_number</t>
         </is>
       </c>
-      <c r="D66" s="9" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>转让人地址
 transferor_address</t>
         </is>
       </c>
-      <c r="E66" s="9" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>受让人
 transferee_name</t>
         </is>
       </c>
-      <c r="F66" s="9" t="inlineStr">
+      <c r="F66" s="2" t="inlineStr">
         <is>
           <t>受让人证件/注册号
 transferee_id_number</t>
         </is>
       </c>
-      <c r="G66" s="9" t="inlineStr">
+      <c r="G66" s="2" t="inlineStr">
         <is>
           <t>受让人地址
 transferee_address</t>
         </is>
       </c>
-      <c r="H66" s="9" t="inlineStr">
+      <c r="H66" s="2" t="inlineStr">
         <is>
           <t>转让股数
 shares_transferred</t>
         </is>
       </c>
-      <c r="I66" s="9" t="inlineStr">
+      <c r="I66" s="2" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="J66" s="9" t="inlineStr">
+      <c r="J66" s="2" t="inlineStr">
         <is>
           <t>转让日期
 transfer_date</t>
         </is>
       </c>
-      <c r="K66" s="9" t="inlineStr">
+      <c r="K66" s="2" t="inlineStr">
         <is>
           <t>对价口径
 consideration_basis</t>
         </is>
       </c>
-      <c r="L66" s="9" t="inlineStr">
+      <c r="L66" s="2" t="inlineStr">
         <is>
           <t>对价金额
 consideration_amount</t>
         </is>
       </c>
-      <c r="M66" s="9" t="inlineStr">
+      <c r="M66" s="2" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="N66" s="9" t="inlineStr">
+      <c r="N66" s="2" t="inlineStr">
         <is>
           <t>旧证书号
 old_certificate_no</t>
         </is>
       </c>
-      <c r="O66" s="9" t="inlineStr">
+      <c r="O66" s="2" t="inlineStr">
         <is>
           <t>新证书号
 new_certificate_no</t>
         </is>
       </c>
-      <c r="P66" s="9" t="inlineStr">
+      <c r="P66" s="2" t="inlineStr">
         <is>
           <t>转让人剩余股数
 transferor_remaining_shares</t>
         </is>
       </c>
-      <c r="Q66" s="9" t="inlineStr">
+      <c r="Q66" s="2" t="inlineStr">
         <is>
           <t>是否生成新证书
 generate_new_certificate</t>
         </is>
       </c>
-      <c r="R66" s="9" t="inlineStr">
+      <c r="R66" s="2" t="inlineStr">
         <is>
           <t>印花税复核
 stamp_duty_review</t>
         </is>
       </c>
-      <c r="S66" s="9" t="inlineStr">
+      <c r="S66" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -1955,291 +1936,291 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="12" t="inlineStr"/>
-      <c r="B67" s="12" t="inlineStr"/>
-      <c r="C67" s="12" t="inlineStr"/>
-      <c r="D67" s="12" t="inlineStr"/>
-      <c r="E67" s="12" t="inlineStr"/>
-      <c r="F67" s="12" t="inlineStr"/>
-      <c r="G67" s="12" t="inlineStr"/>
-      <c r="H67" s="12" t="inlineStr"/>
-      <c r="I67" s="12" t="inlineStr"/>
-      <c r="J67" s="12" t="inlineStr"/>
-      <c r="K67" s="12" t="inlineStr"/>
-      <c r="L67" s="12" t="inlineStr"/>
-      <c r="M67" s="12" t="inlineStr"/>
-      <c r="N67" s="12" t="inlineStr"/>
-      <c r="O67" s="12" t="inlineStr"/>
-      <c r="P67" s="12" t="inlineStr"/>
-      <c r="Q67" s="12" t="inlineStr"/>
-      <c r="R67" s="12" t="inlineStr"/>
-      <c r="S67" s="12" t="inlineStr"/>
+      <c r="A67" s="5" t="inlineStr"/>
+      <c r="B67" s="5" t="inlineStr"/>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr"/>
+      <c r="E67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="5" t="inlineStr"/>
+      <c r="I67" s="5" t="inlineStr"/>
+      <c r="J67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="inlineStr"/>
+      <c r="L67" s="5" t="inlineStr"/>
+      <c r="M67" s="5" t="inlineStr"/>
+      <c r="N67" s="5" t="inlineStr"/>
+      <c r="O67" s="5" t="inlineStr"/>
+      <c r="P67" s="5" t="inlineStr"/>
+      <c r="Q67" s="5" t="inlineStr"/>
+      <c r="R67" s="5" t="inlineStr"/>
+      <c r="S67" s="5" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="12" t="inlineStr"/>
-      <c r="B68" s="12" t="inlineStr"/>
-      <c r="C68" s="12" t="inlineStr"/>
-      <c r="D68" s="12" t="inlineStr"/>
-      <c r="E68" s="12" t="inlineStr"/>
-      <c r="F68" s="12" t="inlineStr"/>
-      <c r="G68" s="12" t="inlineStr"/>
-      <c r="H68" s="12" t="inlineStr"/>
-      <c r="I68" s="12" t="inlineStr"/>
-      <c r="J68" s="12" t="inlineStr"/>
-      <c r="K68" s="12" t="inlineStr"/>
-      <c r="L68" s="12" t="inlineStr"/>
-      <c r="M68" s="12" t="inlineStr"/>
-      <c r="N68" s="12" t="inlineStr"/>
-      <c r="O68" s="12" t="inlineStr"/>
-      <c r="P68" s="12" t="inlineStr"/>
-      <c r="Q68" s="12" t="inlineStr"/>
-      <c r="R68" s="12" t="inlineStr"/>
-      <c r="S68" s="12" t="inlineStr"/>
+      <c r="A68" s="5" t="inlineStr"/>
+      <c r="B68" s="5" t="inlineStr"/>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr"/>
+      <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="5" t="inlineStr"/>
+      <c r="J68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr"/>
+      <c r="M68" s="5" t="inlineStr"/>
+      <c r="N68" s="5" t="inlineStr"/>
+      <c r="O68" s="5" t="inlineStr"/>
+      <c r="P68" s="5" t="inlineStr"/>
+      <c r="Q68" s="5" t="inlineStr"/>
+      <c r="R68" s="5" t="inlineStr"/>
+      <c r="S68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="12" t="inlineStr"/>
-      <c r="B69" s="12" t="inlineStr"/>
-      <c r="C69" s="12" t="inlineStr"/>
-      <c r="D69" s="12" t="inlineStr"/>
-      <c r="E69" s="12" t="inlineStr"/>
-      <c r="F69" s="12" t="inlineStr"/>
-      <c r="G69" s="12" t="inlineStr"/>
-      <c r="H69" s="12" t="inlineStr"/>
-      <c r="I69" s="12" t="inlineStr"/>
-      <c r="J69" s="12" t="inlineStr"/>
-      <c r="K69" s="12" t="inlineStr"/>
-      <c r="L69" s="12" t="inlineStr"/>
-      <c r="M69" s="12" t="inlineStr"/>
-      <c r="N69" s="12" t="inlineStr"/>
-      <c r="O69" s="12" t="inlineStr"/>
-      <c r="P69" s="12" t="inlineStr"/>
-      <c r="Q69" s="12" t="inlineStr"/>
-      <c r="R69" s="12" t="inlineStr"/>
-      <c r="S69" s="12" t="inlineStr"/>
+      <c r="A69" s="5" t="inlineStr"/>
+      <c r="B69" s="5" t="inlineStr"/>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr"/>
+      <c r="E69" s="5" t="inlineStr"/>
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="5" t="inlineStr"/>
+      <c r="I69" s="5" t="inlineStr"/>
+      <c r="J69" s="5" t="inlineStr"/>
+      <c r="K69" s="5" t="inlineStr"/>
+      <c r="L69" s="5" t="inlineStr"/>
+      <c r="M69" s="5" t="inlineStr"/>
+      <c r="N69" s="5" t="inlineStr"/>
+      <c r="O69" s="5" t="inlineStr"/>
+      <c r="P69" s="5" t="inlineStr"/>
+      <c r="Q69" s="5" t="inlineStr"/>
+      <c r="R69" s="5" t="inlineStr"/>
+      <c r="S69" s="5" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="12" t="inlineStr"/>
-      <c r="B70" s="12" t="inlineStr"/>
-      <c r="C70" s="12" t="inlineStr"/>
-      <c r="D70" s="12" t="inlineStr"/>
-      <c r="E70" s="12" t="inlineStr"/>
-      <c r="F70" s="12" t="inlineStr"/>
-      <c r="G70" s="12" t="inlineStr"/>
-      <c r="H70" s="12" t="inlineStr"/>
-      <c r="I70" s="12" t="inlineStr"/>
-      <c r="J70" s="12" t="inlineStr"/>
-      <c r="K70" s="12" t="inlineStr"/>
-      <c r="L70" s="12" t="inlineStr"/>
-      <c r="M70" s="12" t="inlineStr"/>
-      <c r="N70" s="12" t="inlineStr"/>
-      <c r="O70" s="12" t="inlineStr"/>
-      <c r="P70" s="12" t="inlineStr"/>
-      <c r="Q70" s="12" t="inlineStr"/>
-      <c r="R70" s="12" t="inlineStr"/>
-      <c r="S70" s="12" t="inlineStr"/>
+      <c r="A70" s="5" t="inlineStr"/>
+      <c r="B70" s="5" t="inlineStr"/>
+      <c r="C70" s="5" t="inlineStr"/>
+      <c r="D70" s="5" t="inlineStr"/>
+      <c r="E70" s="5" t="inlineStr"/>
+      <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="5" t="inlineStr"/>
+      <c r="H70" s="5" t="inlineStr"/>
+      <c r="I70" s="5" t="inlineStr"/>
+      <c r="J70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="inlineStr"/>
+      <c r="L70" s="5" t="inlineStr"/>
+      <c r="M70" s="5" t="inlineStr"/>
+      <c r="N70" s="5" t="inlineStr"/>
+      <c r="O70" s="5" t="inlineStr"/>
+      <c r="P70" s="5" t="inlineStr"/>
+      <c r="Q70" s="5" t="inlineStr"/>
+      <c r="R70" s="5" t="inlineStr"/>
+      <c r="S70" s="5" t="inlineStr"/>
     </row>
     <row r="71">
-      <c r="A71" s="12" t="inlineStr"/>
-      <c r="B71" s="12" t="inlineStr"/>
-      <c r="C71" s="12" t="inlineStr"/>
-      <c r="D71" s="12" t="inlineStr"/>
-      <c r="E71" s="12" t="inlineStr"/>
-      <c r="F71" s="12" t="inlineStr"/>
-      <c r="G71" s="12" t="inlineStr"/>
-      <c r="H71" s="12" t="inlineStr"/>
-      <c r="I71" s="12" t="inlineStr"/>
-      <c r="J71" s="12" t="inlineStr"/>
-      <c r="K71" s="12" t="inlineStr"/>
-      <c r="L71" s="12" t="inlineStr"/>
-      <c r="M71" s="12" t="inlineStr"/>
-      <c r="N71" s="12" t="inlineStr"/>
-      <c r="O71" s="12" t="inlineStr"/>
-      <c r="P71" s="12" t="inlineStr"/>
-      <c r="Q71" s="12" t="inlineStr"/>
-      <c r="R71" s="12" t="inlineStr"/>
-      <c r="S71" s="12" t="inlineStr"/>
+      <c r="A71" s="5" t="inlineStr"/>
+      <c r="B71" s="5" t="inlineStr"/>
+      <c r="C71" s="5" t="inlineStr"/>
+      <c r="D71" s="5" t="inlineStr"/>
+      <c r="E71" s="5" t="inlineStr"/>
+      <c r="F71" s="5" t="inlineStr"/>
+      <c r="G71" s="5" t="inlineStr"/>
+      <c r="H71" s="5" t="inlineStr"/>
+      <c r="I71" s="5" t="inlineStr"/>
+      <c r="J71" s="5" t="inlineStr"/>
+      <c r="K71" s="5" t="inlineStr"/>
+      <c r="L71" s="5" t="inlineStr"/>
+      <c r="M71" s="5" t="inlineStr"/>
+      <c r="N71" s="5" t="inlineStr"/>
+      <c r="O71" s="5" t="inlineStr"/>
+      <c r="P71" s="5" t="inlineStr"/>
+      <c r="Q71" s="5" t="inlineStr"/>
+      <c r="R71" s="5" t="inlineStr"/>
+      <c r="S71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="inlineStr"/>
-      <c r="B72" s="12" t="inlineStr"/>
-      <c r="C72" s="12" t="inlineStr"/>
-      <c r="D72" s="12" t="inlineStr"/>
-      <c r="E72" s="12" t="inlineStr"/>
-      <c r="F72" s="12" t="inlineStr"/>
-      <c r="G72" s="12" t="inlineStr"/>
-      <c r="H72" s="12" t="inlineStr"/>
-      <c r="I72" s="12" t="inlineStr"/>
-      <c r="J72" s="12" t="inlineStr"/>
-      <c r="K72" s="12" t="inlineStr"/>
-      <c r="L72" s="12" t="inlineStr"/>
-      <c r="M72" s="12" t="inlineStr"/>
-      <c r="N72" s="12" t="inlineStr"/>
-      <c r="O72" s="12" t="inlineStr"/>
-      <c r="P72" s="12" t="inlineStr"/>
-      <c r="Q72" s="12" t="inlineStr"/>
-      <c r="R72" s="12" t="inlineStr"/>
-      <c r="S72" s="12" t="inlineStr"/>
+      <c r="A72" s="5" t="inlineStr"/>
+      <c r="B72" s="5" t="inlineStr"/>
+      <c r="C72" s="5" t="inlineStr"/>
+      <c r="D72" s="5" t="inlineStr"/>
+      <c r="E72" s="5" t="inlineStr"/>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="5" t="inlineStr"/>
+      <c r="H72" s="5" t="inlineStr"/>
+      <c r="I72" s="5" t="inlineStr"/>
+      <c r="J72" s="5" t="inlineStr"/>
+      <c r="K72" s="5" t="inlineStr"/>
+      <c r="L72" s="5" t="inlineStr"/>
+      <c r="M72" s="5" t="inlineStr"/>
+      <c r="N72" s="5" t="inlineStr"/>
+      <c r="O72" s="5" t="inlineStr"/>
+      <c r="P72" s="5" t="inlineStr"/>
+      <c r="Q72" s="5" t="inlineStr"/>
+      <c r="R72" s="5" t="inlineStr"/>
+      <c r="S72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
-      <c r="A73" s="12" t="inlineStr"/>
-      <c r="B73" s="12" t="inlineStr"/>
-      <c r="C73" s="12" t="inlineStr"/>
-      <c r="D73" s="12" t="inlineStr"/>
-      <c r="E73" s="12" t="inlineStr"/>
-      <c r="F73" s="12" t="inlineStr"/>
-      <c r="G73" s="12" t="inlineStr"/>
-      <c r="H73" s="12" t="inlineStr"/>
-      <c r="I73" s="12" t="inlineStr"/>
-      <c r="J73" s="12" t="inlineStr"/>
-      <c r="K73" s="12" t="inlineStr"/>
-      <c r="L73" s="12" t="inlineStr"/>
-      <c r="M73" s="12" t="inlineStr"/>
-      <c r="N73" s="12" t="inlineStr"/>
-      <c r="O73" s="12" t="inlineStr"/>
-      <c r="P73" s="12" t="inlineStr"/>
-      <c r="Q73" s="12" t="inlineStr"/>
-      <c r="R73" s="12" t="inlineStr"/>
-      <c r="S73" s="12" t="inlineStr"/>
+      <c r="A73" s="5" t="inlineStr"/>
+      <c r="B73" s="5" t="inlineStr"/>
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr"/>
+      <c r="E73" s="5" t="inlineStr"/>
+      <c r="F73" s="5" t="inlineStr"/>
+      <c r="G73" s="5" t="inlineStr"/>
+      <c r="H73" s="5" t="inlineStr"/>
+      <c r="I73" s="5" t="inlineStr"/>
+      <c r="J73" s="5" t="inlineStr"/>
+      <c r="K73" s="5" t="inlineStr"/>
+      <c r="L73" s="5" t="inlineStr"/>
+      <c r="M73" s="5" t="inlineStr"/>
+      <c r="N73" s="5" t="inlineStr"/>
+      <c r="O73" s="5" t="inlineStr"/>
+      <c r="P73" s="5" t="inlineStr"/>
+      <c r="Q73" s="5" t="inlineStr"/>
+      <c r="R73" s="5" t="inlineStr"/>
+      <c r="S73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="inlineStr"/>
-      <c r="B74" s="12" t="inlineStr"/>
-      <c r="C74" s="12" t="inlineStr"/>
-      <c r="D74" s="12" t="inlineStr"/>
-      <c r="E74" s="12" t="inlineStr"/>
-      <c r="F74" s="12" t="inlineStr"/>
-      <c r="G74" s="12" t="inlineStr"/>
-      <c r="H74" s="12" t="inlineStr"/>
-      <c r="I74" s="12" t="inlineStr"/>
-      <c r="J74" s="12" t="inlineStr"/>
-      <c r="K74" s="12" t="inlineStr"/>
-      <c r="L74" s="12" t="inlineStr"/>
-      <c r="M74" s="12" t="inlineStr"/>
-      <c r="N74" s="12" t="inlineStr"/>
-      <c r="O74" s="12" t="inlineStr"/>
-      <c r="P74" s="12" t="inlineStr"/>
-      <c r="Q74" s="12" t="inlineStr"/>
-      <c r="R74" s="12" t="inlineStr"/>
-      <c r="S74" s="12" t="inlineStr"/>
+      <c r="A74" s="5" t="inlineStr"/>
+      <c r="B74" s="5" t="inlineStr"/>
+      <c r="C74" s="5" t="inlineStr"/>
+      <c r="D74" s="5" t="inlineStr"/>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr"/>
+      <c r="H74" s="5" t="inlineStr"/>
+      <c r="I74" s="5" t="inlineStr"/>
+      <c r="J74" s="5" t="inlineStr"/>
+      <c r="K74" s="5" t="inlineStr"/>
+      <c r="L74" s="5" t="inlineStr"/>
+      <c r="M74" s="5" t="inlineStr"/>
+      <c r="N74" s="5" t="inlineStr"/>
+      <c r="O74" s="5" t="inlineStr"/>
+      <c r="P74" s="5" t="inlineStr"/>
+      <c r="Q74" s="5" t="inlineStr"/>
+      <c r="R74" s="5" t="inlineStr"/>
+      <c r="S74" s="5" t="inlineStr"/>
     </row>
     <row r="75"/>
     <row r="76">
-      <c r="A76" s="14" t="inlineStr">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>增资配股</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="9" t="inlineStr">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B77" s="9" t="inlineStr">
+      <c r="B77" s="2" t="inlineStr">
         <is>
           <t>认购人
 allottee_name</t>
         </is>
       </c>
-      <c r="C77" s="9" t="inlineStr">
+      <c r="C77" s="2" t="inlineStr">
         <is>
           <t>认购人证件/注册号
 allottee_id_number</t>
         </is>
       </c>
-      <c r="D77" s="9" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>认购人地址
 allottee_address</t>
         </is>
       </c>
-      <c r="E77" s="9" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr">
         <is>
           <t>配发股数
 shares_allotted</t>
         </is>
       </c>
-      <c r="F77" s="9" t="inlineStr">
+      <c r="F77" s="2" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="G77" s="9" t="inlineStr">
+      <c r="G77" s="2" t="inlineStr">
         <is>
           <t>本次已发行股本
 issued_share_capital</t>
         </is>
       </c>
-      <c r="H77" s="9" t="inlineStr">
+      <c r="H77" s="2" t="inlineStr">
         <is>
           <t>每股实缴
 amount_paid_per_share</t>
         </is>
       </c>
-      <c r="I77" s="9" t="inlineStr">
+      <c r="I77" s="2" t="inlineStr">
         <is>
           <t>本次实缴资本
 total_paid</t>
         </is>
       </c>
-      <c r="J77" s="9" t="inlineStr">
+      <c r="J77" s="2" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="K77" s="9" t="inlineStr">
+      <c r="K77" s="2" t="inlineStr">
         <is>
           <t>配股日期
 allotment_date</t>
         </is>
       </c>
-      <c r="L77" s="9" t="inlineStr">
+      <c r="L77" s="2" t="inlineStr">
         <is>
           <t>授权日期
 authority_date</t>
         </is>
       </c>
-      <c r="M77" s="9" t="inlineStr">
+      <c r="M77" s="2" t="inlineStr">
         <is>
           <t>是否 Form 24
 form24_required</t>
         </is>
       </c>
-      <c r="N77" s="9" t="inlineStr">
+      <c r="N77" s="2" t="inlineStr">
         <is>
           <t>证书号
 certificate_no</t>
         </is>
       </c>
-      <c r="O77" s="9" t="inlineStr">
+      <c r="O77" s="2" t="inlineStr">
         <is>
           <t>是否生成证书
 generate_certificate</t>
         </is>
       </c>
-      <c r="P77" s="9" t="inlineStr">
+      <c r="P77" s="2" t="inlineStr">
         <is>
           <t>配股后总股数
 post_allotment_total_shares</t>
         </is>
       </c>
-      <c r="Q77" s="9" t="inlineStr">
+      <c r="Q77" s="2" t="inlineStr">
         <is>
           <t>配股后已发行股本
 post_allotment_issued_share_capital</t>
         </is>
       </c>
-      <c r="R77" s="9" t="inlineStr">
+      <c r="R77" s="2" t="inlineStr">
         <is>
           <t>配股后实缴资本
 post_allotment_paid_up_capital</t>
         </is>
       </c>
-      <c r="S77" s="9" t="inlineStr">
+      <c r="S77" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
@@ -2247,172 +2228,172 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="12" t="inlineStr"/>
-      <c r="B78" s="12" t="inlineStr"/>
-      <c r="C78" s="12" t="inlineStr"/>
-      <c r="D78" s="12" t="inlineStr"/>
-      <c r="E78" s="12" t="inlineStr"/>
-      <c r="F78" s="12" t="inlineStr"/>
-      <c r="G78" s="12" t="inlineStr"/>
-      <c r="H78" s="12" t="inlineStr"/>
-      <c r="I78" s="12" t="inlineStr"/>
-      <c r="J78" s="12" t="inlineStr"/>
-      <c r="K78" s="12" t="inlineStr"/>
-      <c r="L78" s="12" t="inlineStr"/>
-      <c r="M78" s="12" t="inlineStr"/>
-      <c r="N78" s="12" t="inlineStr"/>
-      <c r="O78" s="12" t="inlineStr"/>
-      <c r="P78" s="12" t="inlineStr"/>
-      <c r="Q78" s="12" t="inlineStr"/>
-      <c r="R78" s="12" t="inlineStr"/>
-      <c r="S78" s="12" t="inlineStr"/>
+      <c r="A78" s="5" t="inlineStr"/>
+      <c r="B78" s="5" t="inlineStr"/>
+      <c r="C78" s="5" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr"/>
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="5" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
+      <c r="N78" s="5" t="inlineStr"/>
+      <c r="O78" s="5" t="inlineStr"/>
+      <c r="P78" s="5" t="inlineStr"/>
+      <c r="Q78" s="5" t="inlineStr"/>
+      <c r="R78" s="5" t="inlineStr"/>
+      <c r="S78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="12" t="inlineStr"/>
-      <c r="B79" s="12" t="inlineStr"/>
-      <c r="C79" s="12" t="inlineStr"/>
-      <c r="D79" s="12" t="inlineStr"/>
-      <c r="E79" s="12" t="inlineStr"/>
-      <c r="F79" s="12" t="inlineStr"/>
-      <c r="G79" s="12" t="inlineStr"/>
-      <c r="H79" s="12" t="inlineStr"/>
-      <c r="I79" s="12" t="inlineStr"/>
-      <c r="J79" s="12" t="inlineStr"/>
-      <c r="K79" s="12" t="inlineStr"/>
-      <c r="L79" s="12" t="inlineStr"/>
-      <c r="M79" s="12" t="inlineStr"/>
-      <c r="N79" s="12" t="inlineStr"/>
-      <c r="O79" s="12" t="inlineStr"/>
-      <c r="P79" s="12" t="inlineStr"/>
-      <c r="Q79" s="12" t="inlineStr"/>
-      <c r="R79" s="12" t="inlineStr"/>
-      <c r="S79" s="12" t="inlineStr"/>
+      <c r="A79" s="5" t="inlineStr"/>
+      <c r="B79" s="5" t="inlineStr"/>
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr"/>
+      <c r="E79" s="5" t="inlineStr"/>
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr"/>
+      <c r="I79" s="5" t="inlineStr"/>
+      <c r="J79" s="5" t="inlineStr"/>
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
+      <c r="N79" s="5" t="inlineStr"/>
+      <c r="O79" s="5" t="inlineStr"/>
+      <c r="P79" s="5" t="inlineStr"/>
+      <c r="Q79" s="5" t="inlineStr"/>
+      <c r="R79" s="5" t="inlineStr"/>
+      <c r="S79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="12" t="inlineStr"/>
-      <c r="B80" s="12" t="inlineStr"/>
-      <c r="C80" s="12" t="inlineStr"/>
-      <c r="D80" s="12" t="inlineStr"/>
-      <c r="E80" s="12" t="inlineStr"/>
-      <c r="F80" s="12" t="inlineStr"/>
-      <c r="G80" s="12" t="inlineStr"/>
-      <c r="H80" s="12" t="inlineStr"/>
-      <c r="I80" s="12" t="inlineStr"/>
-      <c r="J80" s="12" t="inlineStr"/>
-      <c r="K80" s="12" t="inlineStr"/>
-      <c r="L80" s="12" t="inlineStr"/>
-      <c r="M80" s="12" t="inlineStr"/>
-      <c r="N80" s="12" t="inlineStr"/>
-      <c r="O80" s="12" t="inlineStr"/>
-      <c r="P80" s="12" t="inlineStr"/>
-      <c r="Q80" s="12" t="inlineStr"/>
-      <c r="R80" s="12" t="inlineStr"/>
-      <c r="S80" s="12" t="inlineStr"/>
+      <c r="A80" s="5" t="inlineStr"/>
+      <c r="B80" s="5" t="inlineStr"/>
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr"/>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="5" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
+      <c r="N80" s="5" t="inlineStr"/>
+      <c r="O80" s="5" t="inlineStr"/>
+      <c r="P80" s="5" t="inlineStr"/>
+      <c r="Q80" s="5" t="inlineStr"/>
+      <c r="R80" s="5" t="inlineStr"/>
+      <c r="S80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
-      <c r="A81" s="12" t="inlineStr"/>
-      <c r="B81" s="12" t="inlineStr"/>
-      <c r="C81" s="12" t="inlineStr"/>
-      <c r="D81" s="12" t="inlineStr"/>
-      <c r="E81" s="12" t="inlineStr"/>
-      <c r="F81" s="12" t="inlineStr"/>
-      <c r="G81" s="12" t="inlineStr"/>
-      <c r="H81" s="12" t="inlineStr"/>
-      <c r="I81" s="12" t="inlineStr"/>
-      <c r="J81" s="12" t="inlineStr"/>
-      <c r="K81" s="12" t="inlineStr"/>
-      <c r="L81" s="12" t="inlineStr"/>
-      <c r="M81" s="12" t="inlineStr"/>
-      <c r="N81" s="12" t="inlineStr"/>
-      <c r="O81" s="12" t="inlineStr"/>
-      <c r="P81" s="12" t="inlineStr"/>
-      <c r="Q81" s="12" t="inlineStr"/>
-      <c r="R81" s="12" t="inlineStr"/>
-      <c r="S81" s="12" t="inlineStr"/>
+      <c r="A81" s="5" t="inlineStr"/>
+      <c r="B81" s="5" t="inlineStr"/>
+      <c r="C81" s="5" t="inlineStr"/>
+      <c r="D81" s="5" t="inlineStr"/>
+      <c r="E81" s="5" t="inlineStr"/>
+      <c r="F81" s="5" t="inlineStr"/>
+      <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
+      <c r="I81" s="5" t="inlineStr"/>
+      <c r="J81" s="5" t="inlineStr"/>
+      <c r="K81" s="5" t="inlineStr"/>
+      <c r="L81" s="5" t="inlineStr"/>
+      <c r="M81" s="5" t="inlineStr"/>
+      <c r="N81" s="5" t="inlineStr"/>
+      <c r="O81" s="5" t="inlineStr"/>
+      <c r="P81" s="5" t="inlineStr"/>
+      <c r="Q81" s="5" t="inlineStr"/>
+      <c r="R81" s="5" t="inlineStr"/>
+      <c r="S81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="12" t="inlineStr"/>
-      <c r="B82" s="12" t="inlineStr"/>
-      <c r="C82" s="12" t="inlineStr"/>
-      <c r="D82" s="12" t="inlineStr"/>
-      <c r="E82" s="12" t="inlineStr"/>
-      <c r="F82" s="12" t="inlineStr"/>
-      <c r="G82" s="12" t="inlineStr"/>
-      <c r="H82" s="12" t="inlineStr"/>
-      <c r="I82" s="12" t="inlineStr"/>
-      <c r="J82" s="12" t="inlineStr"/>
-      <c r="K82" s="12" t="inlineStr"/>
-      <c r="L82" s="12" t="inlineStr"/>
-      <c r="M82" s="12" t="inlineStr"/>
-      <c r="N82" s="12" t="inlineStr"/>
-      <c r="O82" s="12" t="inlineStr"/>
-      <c r="P82" s="12" t="inlineStr"/>
-      <c r="Q82" s="12" t="inlineStr"/>
-      <c r="R82" s="12" t="inlineStr"/>
-      <c r="S82" s="12" t="inlineStr"/>
+      <c r="A82" s="5" t="inlineStr"/>
+      <c r="B82" s="5" t="inlineStr"/>
+      <c r="C82" s="5" t="inlineStr"/>
+      <c r="D82" s="5" t="inlineStr"/>
+      <c r="E82" s="5" t="inlineStr"/>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr"/>
+      <c r="H82" s="5" t="inlineStr"/>
+      <c r="I82" s="5" t="inlineStr"/>
+      <c r="J82" s="5" t="inlineStr"/>
+      <c r="K82" s="5" t="inlineStr"/>
+      <c r="L82" s="5" t="inlineStr"/>
+      <c r="M82" s="5" t="inlineStr"/>
+      <c r="N82" s="5" t="inlineStr"/>
+      <c r="O82" s="5" t="inlineStr"/>
+      <c r="P82" s="5" t="inlineStr"/>
+      <c r="Q82" s="5" t="inlineStr"/>
+      <c r="R82" s="5" t="inlineStr"/>
+      <c r="S82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
-      <c r="A83" s="12" t="inlineStr"/>
-      <c r="B83" s="12" t="inlineStr"/>
-      <c r="C83" s="12" t="inlineStr"/>
-      <c r="D83" s="12" t="inlineStr"/>
-      <c r="E83" s="12" t="inlineStr"/>
-      <c r="F83" s="12" t="inlineStr"/>
-      <c r="G83" s="12" t="inlineStr"/>
-      <c r="H83" s="12" t="inlineStr"/>
-      <c r="I83" s="12" t="inlineStr"/>
-      <c r="J83" s="12" t="inlineStr"/>
-      <c r="K83" s="12" t="inlineStr"/>
-      <c r="L83" s="12" t="inlineStr"/>
-      <c r="M83" s="12" t="inlineStr"/>
-      <c r="N83" s="12" t="inlineStr"/>
-      <c r="O83" s="12" t="inlineStr"/>
-      <c r="P83" s="12" t="inlineStr"/>
-      <c r="Q83" s="12" t="inlineStr"/>
-      <c r="R83" s="12" t="inlineStr"/>
-      <c r="S83" s="12" t="inlineStr"/>
+      <c r="A83" s="5" t="inlineStr"/>
+      <c r="B83" s="5" t="inlineStr"/>
+      <c r="C83" s="5" t="inlineStr"/>
+      <c r="D83" s="5" t="inlineStr"/>
+      <c r="E83" s="5" t="inlineStr"/>
+      <c r="F83" s="5" t="inlineStr"/>
+      <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="5" t="inlineStr"/>
+      <c r="I83" s="5" t="inlineStr"/>
+      <c r="J83" s="5" t="inlineStr"/>
+      <c r="K83" s="5" t="inlineStr"/>
+      <c r="L83" s="5" t="inlineStr"/>
+      <c r="M83" s="5" t="inlineStr"/>
+      <c r="N83" s="5" t="inlineStr"/>
+      <c r="O83" s="5" t="inlineStr"/>
+      <c r="P83" s="5" t="inlineStr"/>
+      <c r="Q83" s="5" t="inlineStr"/>
+      <c r="R83" s="5" t="inlineStr"/>
+      <c r="S83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="inlineStr"/>
-      <c r="B84" s="12" t="inlineStr"/>
-      <c r="C84" s="12" t="inlineStr"/>
-      <c r="D84" s="12" t="inlineStr"/>
-      <c r="E84" s="12" t="inlineStr"/>
-      <c r="F84" s="12" t="inlineStr"/>
-      <c r="G84" s="12" t="inlineStr"/>
-      <c r="H84" s="12" t="inlineStr"/>
-      <c r="I84" s="12" t="inlineStr"/>
-      <c r="J84" s="12" t="inlineStr"/>
-      <c r="K84" s="12" t="inlineStr"/>
-      <c r="L84" s="12" t="inlineStr"/>
-      <c r="M84" s="12" t="inlineStr"/>
-      <c r="N84" s="12" t="inlineStr"/>
-      <c r="O84" s="12" t="inlineStr"/>
-      <c r="P84" s="12" t="inlineStr"/>
-      <c r="Q84" s="12" t="inlineStr"/>
-      <c r="R84" s="12" t="inlineStr"/>
-      <c r="S84" s="12" t="inlineStr"/>
+      <c r="A84" s="5" t="inlineStr"/>
+      <c r="B84" s="5" t="inlineStr"/>
+      <c r="C84" s="5" t="inlineStr"/>
+      <c r="D84" s="5" t="inlineStr"/>
+      <c r="E84" s="5" t="inlineStr"/>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="5" t="inlineStr"/>
+      <c r="H84" s="5" t="inlineStr"/>
+      <c r="I84" s="5" t="inlineStr"/>
+      <c r="J84" s="5" t="inlineStr"/>
+      <c r="K84" s="5" t="inlineStr"/>
+      <c r="L84" s="5" t="inlineStr"/>
+      <c r="M84" s="5" t="inlineStr"/>
+      <c r="N84" s="5" t="inlineStr"/>
+      <c r="O84" s="5" t="inlineStr"/>
+      <c r="P84" s="5" t="inlineStr"/>
+      <c r="Q84" s="5" t="inlineStr"/>
+      <c r="R84" s="5" t="inlineStr"/>
+      <c r="S84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
-      <c r="A85" s="12" t="inlineStr"/>
-      <c r="B85" s="12" t="inlineStr"/>
-      <c r="C85" s="12" t="inlineStr"/>
-      <c r="D85" s="12" t="inlineStr"/>
-      <c r="E85" s="12" t="inlineStr"/>
-      <c r="F85" s="12" t="inlineStr"/>
-      <c r="G85" s="12" t="inlineStr"/>
-      <c r="H85" s="12" t="inlineStr"/>
-      <c r="I85" s="12" t="inlineStr"/>
-      <c r="J85" s="12" t="inlineStr"/>
-      <c r="K85" s="12" t="inlineStr"/>
-      <c r="L85" s="12" t="inlineStr"/>
-      <c r="M85" s="12" t="inlineStr"/>
-      <c r="N85" s="12" t="inlineStr"/>
-      <c r="O85" s="12" t="inlineStr"/>
-      <c r="P85" s="12" t="inlineStr"/>
-      <c r="Q85" s="12" t="inlineStr"/>
-      <c r="R85" s="12" t="inlineStr"/>
-      <c r="S85" s="12" t="inlineStr"/>
+      <c r="A85" s="5" t="inlineStr"/>
+      <c r="B85" s="5" t="inlineStr"/>
+      <c r="C85" s="5" t="inlineStr"/>
+      <c r="D85" s="5" t="inlineStr"/>
+      <c r="E85" s="5" t="inlineStr"/>
+      <c r="F85" s="5" t="inlineStr"/>
+      <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="5" t="inlineStr"/>
+      <c r="I85" s="5" t="inlineStr"/>
+      <c r="J85" s="5" t="inlineStr"/>
+      <c r="K85" s="5" t="inlineStr"/>
+      <c r="L85" s="5" t="inlineStr"/>
+      <c r="M85" s="5" t="inlineStr"/>
+      <c r="N85" s="5" t="inlineStr"/>
+      <c r="O85" s="5" t="inlineStr"/>
+      <c r="P85" s="5" t="inlineStr"/>
+      <c r="Q85" s="5" t="inlineStr"/>
+      <c r="R85" s="5" t="inlineStr"/>
+      <c r="S85" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2496,7 +2477,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>快速年审 Annual Review - 常用默认值已内置</t>
         </is>
@@ -2504,764 +2485,764 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>项目</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>English</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>field_key</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>填写内容 / Value</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>是否做年审</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Annual review required</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>annual_review_required</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr"/>
-      <c r="E4" s="10" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>财年结束日</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Financial year end</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>fye_date</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr"/>
-      <c r="E5" s="10" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>必填</t>
         </is>
       </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>DD/MM/YYYY。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>AGM 日期</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>AGM date</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>agm_date</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr"/>
-      <c r="E6" s="10" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>建议填</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>留空后续可由系统按规则推定。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>AGM 时间</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>AGM time</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>agm_time</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>10.00 a.m.</t>
         </is>
       </c>
-      <c r="E7" s="10" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>通常不用改。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>AGM 地点</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>AGM place</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>agm_place</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>默认注册地址</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>留空默认当前注册地址。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>年审方式</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>AGM route</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Annual review method</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>agm_route</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>ordinary_agm</t>
         </is>
       </c>
-      <c r="E9" s="10" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>ordinary_agm / exempt_private_company / dormant_company / manual。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>财报状态</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Accounts status</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>accounts_status</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>non_dormant</t>
-        </is>
-      </c>
-      <c r="E10" s="10" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>常用</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>non_dormant / dormant / unaudited / audited。</t>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>active / dormant / audited；通常填 active，休眠才填 dormant，已审计才填 audited。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t>公司活动状态</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Company activity status</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>company_activity_status</t>
         </is>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="E11" s="10" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Active / Dormant；留空按 Active。</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t>是否 ACRA 休眠相关公司</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>ACRA dormant relevant company</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>acra_dormant_relevant_company</t>
         </is>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E12" s="10" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Auto / Yes / No；休眠公司会影响是否需要财报。</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>资产是否不超过 50 万</t>
         </is>
       </c>
-      <c r="B13" s="10" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Total assets under S$500k</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>total_assets_under_500k</t>
         </is>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E13" s="10" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Auto / Yes / No；用于判断 dormant AGM exemption 风险。</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>是否需要财报</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Financial statements required</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>financial_statements_required</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E14" s="10" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Auto / Yes / No；休眠且符合条件时可 No。</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="10" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>财报类型</t>
         </is>
       </c>
-      <c r="B15" s="10" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Financial statements type</t>
         </is>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>financial_statements_type</t>
         </is>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E15" s="10" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Auto / Unaudited / Audited / Dormant no FS / Management accounts。</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>审计/豁免状态</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Audit exemption status</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>audit_exemption_status</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E16" s="10" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Auto / Small company exempt / Audited / Dormant relevant / Manual review。</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>AGM 状态</t>
         </is>
       </c>
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>AGM status</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>agm_status</t>
         </is>
       </c>
-      <c r="D17" s="12" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>默认 Auto</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Auto / Held AGM / Dispensed with AGM / Exempt from AGM / Written resolutions。</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>IRAS 税务状态</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>IRAS tax status</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>iras_tax_status</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E18" s="10" t="inlineStr">
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Auto / Active / Dormant / Dormant waiver granted / Manual review；只作复核提醒。</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t>财报日期</t>
         </is>
       </c>
-      <c r="B19" s="10" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Financial statement date</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>financial_statement_date</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr"/>
-      <c r="E19" s="10" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>默认 FYE</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>留空默认财年结束日。</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t>董事签字人</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>Director signer</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>director_signer_name</t>
         </is>
       </c>
-      <c r="D20" s="12" t="inlineStr"/>
-      <c r="E20" s="10" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>常用</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
+      <c r="F20" s="6" t="inlineStr">
         <is>
           <t>留空默认首页董事签字人。</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>股东/成员签字人</t>
         </is>
       </c>
-      <c r="B21" s="10" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Shareholder signer</t>
         </is>
       </c>
-      <c r="C21" s="11" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>shareholder_signer_name</t>
         </is>
       </c>
-      <c r="D21" s="12" t="inlineStr"/>
-      <c r="E21" s="10" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
         <is>
           <t>需要股东签署的年审文件使用。</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>AR 授权签字人</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>AR authorised signer</t>
         </is>
       </c>
-      <c r="C22" s="11" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>ar_authorized_signer_name</t>
         </is>
       </c>
-      <c r="D22" s="12" t="inlineStr"/>
-      <c r="E22" s="10" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>默认董事签字人</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="F22" s="6" t="inlineStr">
         <is>
           <t>Annual Return 授权。</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="10" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>董事费</t>
         </is>
       </c>
-      <c r="B23" s="10" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Directors' fee</t>
         </is>
       </c>
-      <c r="C23" s="11" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>directors_fee</t>
         </is>
       </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E23" s="10" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
         <is>
           <t>通常 0。</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>董事薪酬</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Directors' remuneration</t>
         </is>
       </c>
-      <c r="C24" s="11" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>directors_remuneration</t>
         </is>
       </c>
-      <c r="D24" s="12" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="E24" s="10" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="F24" s="6" t="inlineStr">
         <is>
           <t>通常 0。</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Shorter Notice Consent</t>
         </is>
       </c>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Shorter notice consent</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>shorter_notice_consent</t>
         </is>
       </c>
-      <c r="D25" s="12" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Auto</t>
         </is>
       </c>
-      <c r="E25" s="10" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F25" s="13" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
         <is>
           <t>Auto / Yes / No。</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Management Representation Letter</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>MRL</t>
         </is>
       </c>
-      <c r="C26" s="11" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>management_rep_letter</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E26" s="10" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>默认</t>
         </is>
       </c>
-      <c r="F26" s="13" t="inlineStr">
+      <c r="F26" s="6" t="inlineStr">
         <is>
           <t>Yes / No。</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>备注</t>
         </is>
       </c>
-      <c r="B27" s="10" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>remarks</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr"/>
-      <c r="E27" s="10" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
         <is>
           <t>特殊情况写这里。</t>
         </is>
@@ -3279,7 +3260,7 @@
       <formula1>"ordinary_agm,exempt_private_company,dormant_company,written_resolutions,manual"</formula1>
     </dataValidation>
     <dataValidation sqref="D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"non_dormant,dormant,unaudited,audited,manual"</formula1>
+      <formula1>"active,dormant,audited"</formula1>
     </dataValidation>
     <dataValidation sqref="D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Active,Dormant"</formula1>

</xml_diff>

<commit_message>
Simplify M05 annual review flow
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -2663,7 +2663,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>年审方式</t>
+          <t>年审文件方式</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -2688,7 +2688,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>ordinary_agm / exempt_private_company / dormant_company / manual。</t>
+          <t>通常不用改；ordinary_agm=普通 AGM，written_resolutions=书面年审，exempt_private_company/dispensed_with_agm=不召开 AGM。</t>
         </is>
       </c>
     </row>
@@ -2708,19 +2708,15 @@
           <t>accounts_status</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
+      <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>常用</t>
+          <t>核心选项</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>active / dormant / audited；通常填 active，休眠才填 dormant，已审计才填 audited。</t>
+          <t>留空=active；只用 active / dormant / audited。休眠填 dormant，已审计填 audited。</t>
         </is>
       </c>
     </row>
@@ -2740,19 +2736,15 @@
           <t>company_activity_status</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="D11" s="5" t="inlineStr"/>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>默认</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>Active / Dormant；留空按 Active。</t>
+          <t>兼容/复核字段；通常不用填，系统以 accounts_status 为准。</t>
         </is>
       </c>
     </row>
@@ -2772,19 +2764,15 @@
           <t>acra_dormant_relevant_company</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Auto / Yes / No；休眠公司会影响是否需要财报。</t>
+          <t>休眠公司复核用；通常留空。</t>
         </is>
       </c>
     </row>
@@ -2804,19 +2792,15 @@
           <t>total_assets_under_500k</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D13" s="5" t="inlineStr"/>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Auto / Yes / No；用于判断 dormant AGM exemption 风险。</t>
+          <t>休眠公司复核用；通常留空。</t>
         </is>
       </c>
     </row>
@@ -2836,19 +2820,15 @@
           <t>financial_statements_required</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D14" s="5" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>Auto / Yes / No；休眠且符合条件时可 No。</t>
+          <t>通常不用填；系统按 accounts_status 生成相应文件。</t>
         </is>
       </c>
     </row>
@@ -2868,19 +2848,15 @@
           <t>financial_statements_type</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D15" s="5" t="inlineStr"/>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>Auto / Unaudited / Audited / Dormant no FS / Management accounts。</t>
+          <t>兼容字段；通常不用填。普通年审由 accounts_status=active 控制。</t>
         </is>
       </c>
     </row>
@@ -2900,19 +2876,15 @@
           <t>audit_exemption_status</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D16" s="5" t="inlineStr"/>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>Auto / Small company exempt / Audited / Dormant relevant / Manual review。</t>
+          <t>兼容/复核字段；通常不用填。</t>
         </is>
       </c>
     </row>
@@ -2932,19 +2904,15 @@
           <t>agm_status</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D17" s="5" t="inlineStr"/>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>Auto / Held AGM / Dispensed with AGM / Exempt from AGM / Written resolutions。</t>
+          <t>通常不用填；如不召开 AGM，可填 Dispensed with AGM / Exempt from AGM / Written resolutions。</t>
         </is>
       </c>
     </row>
@@ -2964,11 +2932,7 @@
           <t>iras_tax_status</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>Auto</t>
-        </is>
-      </c>
+      <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="3" t="inlineStr">
         <is>
           <t>可空</t>
@@ -2976,7 +2940,7 @@
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>Auto / Active / Dormant / Dormant waiver granted / Manual review；只作复核提醒。</t>
+          <t>只作复核提醒；通常不用填。</t>
         </is>
       </c>
     </row>
@@ -3257,13 +3221,13 @@
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ordinary_agm,exempt_private_company,dormant_company,written_resolutions,manual"</formula1>
+      <formula1>"ordinary_agm,written_resolutions,exempt_private_company,dispensed_with_agm,manual"</formula1>
     </dataValidation>
     <dataValidation sqref="D10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"active,dormant,audited"</formula1>
     </dataValidation>
     <dataValidation sqref="D11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Active,Dormant"</formula1>
+      <formula1>"Auto,Active,Dormant"</formula1>
     </dataValidation>
     <dataValidation sqref="D12" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
@@ -3275,10 +3239,10 @@
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="D15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Auto,Unaudited,Audited,Dormant no FS,Management accounts,Not applicable"</formula1>
+      <formula1>"Auto,Unaudited,Audited,Management accounts,Not applicable"</formula1>
     </dataValidation>
     <dataValidation sqref="D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Auto,Small company exempt,Audited,Dormant relevant,Manual review"</formula1>
+      <formula1>"Auto,Small company exempt,Audited,Manual review"</formula1>
     </dataValidation>
     <dataValidation sqref="D17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Held AGM,Dispensed with AGM,Exempt from AGM,Written resolutions,Manual review"</formula1>

</xml_diff>

<commit_message>
Add M06 strike-off package and polish P2 form UI
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S88"/>
+  <dimension ref="A1:S91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1523,73 +1523,73 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>是否做年审</t>
+          <t>是否注销公司</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Annual review required</t>
+          <t>Strike-off required</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>annual_review_required</t>
+          <t>strike_off_required</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr"/>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>默认 Auto</t>
+          <t>需要时填 Yes</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
+          <t>触发 M06 注销签署包；留空不触发。</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>年审 FYE</t>
+          <t>业务停止日期</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>Annual review FYE</t>
+          <t>Business cessation date</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>fye_date</t>
+          <t>strike_off_cessation_date</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr"/>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>年审时填</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>DD/MM/YYYY。</t>
+          <t>DD/MM/YYYY；留空表示公司自注册后未开展业务。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>AGM 日期</t>
+          <t>注销声明签字董事</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>AGM date</t>
+          <t>Strike-off declaration signer</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>agm_date</t>
+          <t>strike_off_declaration_signer_name</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr"/>
@@ -1600,136 +1600,196 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>DD/MM/YYYY。</t>
+          <t>留空默认第一个董事签字人。</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>年审备注</t>
+          <t>是否做年审</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Annual review remarks</t>
+          <t>Annual review required</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>annual_review_remarks</t>
+          <t>annual_review_required</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr"/>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>可空</t>
+          <t>默认 Auto</t>
         </is>
       </c>
       <c r="F42" s="6" t="inlineStr">
         <is>
-          <t>复杂情况写这里；详细字段可填“快速年审”页。</t>
+          <t>留空/Auto 时，填写 FYE 或 AGM 日期即可生成年审包；填 No 则不生成。</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>备注</t>
+          <t>年审 FYE</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Annual review FYE</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>fye_date</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr"/>
       <c r="E43" s="3" t="inlineStr">
         <is>
+          <t>年审时填</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>DD/MM/YYYY。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>AGM 日期</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>AGM date</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>agm_date</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
           <t>可空</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>DD/MM/YYYY。</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>年审备注</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Annual review remarks</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>annual_review_remarks</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>可空</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>复杂情况写这里；详细字段可填“快速年审”页。</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>可空</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
         <is>
           <t>内部备注，不进正式文件。</t>
         </is>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="7" t="inlineStr">
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
         <is>
           <t>人员任免</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>动作
 action_type</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>是否出辞职信
 resignation_letter</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
         </is>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="5" t="inlineStr"/>
-      <c r="B48" s="5" t="inlineStr"/>
-      <c r="C48" s="5" t="inlineStr"/>
-      <c r="D48" s="5" t="inlineStr"/>
-      <c r="E48" s="5" t="inlineStr"/>
-      <c r="F48" s="5" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr"/>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr"/>
-      <c r="D49" s="5" t="inlineStr"/>
-      <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="5" t="inlineStr"/>
-      <c r="B50" s="5" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr"/>
-      <c r="D50" s="5" t="inlineStr"/>
-      <c r="E50" s="5" t="inlineStr"/>
-      <c r="F50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr"/>
@@ -1771,84 +1831,81 @@
       <c r="E55" s="5" t="inlineStr"/>
       <c r="F55" s="5" t="inlineStr"/>
     </row>
-    <row r="56"/>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr"/>
+      <c r="B56" s="5" t="inlineStr"/>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr"/>
+    </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr"/>
+      <c r="B57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr"/>
+      <c r="B58" s="5" t="inlineStr"/>
+      <c r="C58" s="5" t="inlineStr"/>
+      <c r="D58" s="5" t="inlineStr"/>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="inlineStr"/>
+    </row>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>个人资料变更</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B61" s="2" t="inlineStr">
         <is>
           <t>人员姓名
 target_name</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr">
         <is>
           <t>变更字段
 field_label</t>
         </is>
       </c>
-      <c r="D58" s="2" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>原资料
 old_value</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>新资料
 new_value</t>
         </is>
       </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="F61" s="2" t="inlineStr">
         <is>
           <t>生效日期
 effective_date</t>
         </is>
       </c>
-      <c r="G58" s="2" t="inlineStr">
+      <c r="G61" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
         </is>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr"/>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="5" t="inlineStr"/>
-      <c r="D59" s="5" t="inlineStr"/>
-      <c r="E59" s="5" t="inlineStr"/>
-      <c r="F59" s="5" t="inlineStr"/>
-      <c r="G59" s="5" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr"/>
-      <c r="B60" s="5" t="inlineStr"/>
-      <c r="C60" s="5" t="inlineStr"/>
-      <c r="D60" s="5" t="inlineStr"/>
-      <c r="E60" s="5" t="inlineStr"/>
-      <c r="F60" s="5" t="inlineStr"/>
-      <c r="G60" s="5" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr"/>
-      <c r="B61" s="5" t="inlineStr"/>
-      <c r="C61" s="5" t="inlineStr"/>
-      <c r="D61" s="5" t="inlineStr"/>
-      <c r="E61" s="5" t="inlineStr"/>
-      <c r="F61" s="5" t="inlineStr"/>
-      <c r="G61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr"/>
@@ -1895,192 +1952,156 @@
       <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr"/>
     </row>
-    <row r="67"/>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr"/>
+      <c r="B67" s="5" t="inlineStr"/>
+      <c r="C67" s="5" t="inlineStr"/>
+      <c r="D67" s="5" t="inlineStr"/>
+      <c r="E67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="inlineStr"/>
+      <c r="G67" s="5" t="inlineStr"/>
+    </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
+      <c r="A68" s="5" t="inlineStr"/>
+      <c r="B68" s="5" t="inlineStr"/>
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr"/>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr"/>
+      <c r="B69" s="5" t="inlineStr"/>
+      <c r="C69" s="5" t="inlineStr"/>
+      <c r="D69" s="5" t="inlineStr"/>
+      <c r="E69" s="5" t="inlineStr"/>
+      <c r="F69" s="5" t="inlineStr"/>
+      <c r="G69" s="5" t="inlineStr"/>
+    </row>
+    <row r="70"/>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>股份转让</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="2" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>转让人
 transferor_name</t>
         </is>
       </c>
-      <c r="C69" s="2" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>转让人证件/注册号
 transferor_id_number</t>
         </is>
       </c>
-      <c r="D69" s="2" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>转让人地址
 transferor_address</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr">
         <is>
           <t>受让人
 transferee_name</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr">
+      <c r="F72" s="2" t="inlineStr">
         <is>
           <t>受让人证件/注册号
 transferee_id_number</t>
         </is>
       </c>
-      <c r="G69" s="2" t="inlineStr">
+      <c r="G72" s="2" t="inlineStr">
         <is>
           <t>受让人地址
 transferee_address</t>
         </is>
       </c>
-      <c r="H69" s="2" t="inlineStr">
+      <c r="H72" s="2" t="inlineStr">
         <is>
           <t>转让股数
 shares_transferred</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="J69" s="2" t="inlineStr">
+      <c r="J72" s="2" t="inlineStr">
         <is>
           <t>转让日期
 transfer_date</t>
         </is>
       </c>
-      <c r="K69" s="2" t="inlineStr">
+      <c r="K72" s="2" t="inlineStr">
         <is>
           <t>对价口径
 consideration_basis</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="L72" s="2" t="inlineStr">
         <is>
           <t>对价金额
 consideration_amount</t>
         </is>
       </c>
-      <c r="M69" s="2" t="inlineStr">
+      <c r="M72" s="2" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="N69" s="2" t="inlineStr">
+      <c r="N72" s="2" t="inlineStr">
         <is>
           <t>旧证书号
 old_certificate_no</t>
         </is>
       </c>
-      <c r="O69" s="2" t="inlineStr">
+      <c r="O72" s="2" t="inlineStr">
         <is>
           <t>新证书号
 new_certificate_no</t>
         </is>
       </c>
-      <c r="P69" s="2" t="inlineStr">
+      <c r="P72" s="2" t="inlineStr">
         <is>
           <t>转让人剩余股数
 transferor_remaining_shares</t>
         </is>
       </c>
-      <c r="Q69" s="2" t="inlineStr">
+      <c r="Q72" s="2" t="inlineStr">
         <is>
           <t>是否生成新证书
 generate_new_certificate</t>
         </is>
       </c>
-      <c r="R69" s="2" t="inlineStr">
+      <c r="R72" s="2" t="inlineStr">
         <is>
           <t>印花税复核
 stamp_duty_review</t>
         </is>
       </c>
-      <c r="S69" s="2" t="inlineStr">
+      <c r="S72" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
         </is>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr"/>
-      <c r="B70" s="5" t="inlineStr"/>
-      <c r="C70" s="5" t="inlineStr"/>
-      <c r="D70" s="5" t="inlineStr"/>
-      <c r="E70" s="5" t="inlineStr"/>
-      <c r="F70" s="5" t="inlineStr"/>
-      <c r="G70" s="5" t="inlineStr"/>
-      <c r="H70" s="5" t="inlineStr"/>
-      <c r="I70" s="5" t="inlineStr"/>
-      <c r="J70" s="5" t="inlineStr"/>
-      <c r="K70" s="5" t="inlineStr"/>
-      <c r="L70" s="5" t="inlineStr"/>
-      <c r="M70" s="5" t="inlineStr"/>
-      <c r="N70" s="5" t="inlineStr"/>
-      <c r="O70" s="5" t="inlineStr"/>
-      <c r="P70" s="5" t="inlineStr"/>
-      <c r="Q70" s="5" t="inlineStr"/>
-      <c r="R70" s="5" t="inlineStr"/>
-      <c r="S70" s="5" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr"/>
-      <c r="B71" s="5" t="inlineStr"/>
-      <c r="C71" s="5" t="inlineStr"/>
-      <c r="D71" s="5" t="inlineStr"/>
-      <c r="E71" s="5" t="inlineStr"/>
-      <c r="F71" s="5" t="inlineStr"/>
-      <c r="G71" s="5" t="inlineStr"/>
-      <c r="H71" s="5" t="inlineStr"/>
-      <c r="I71" s="5" t="inlineStr"/>
-      <c r="J71" s="5" t="inlineStr"/>
-      <c r="K71" s="5" t="inlineStr"/>
-      <c r="L71" s="5" t="inlineStr"/>
-      <c r="M71" s="5" t="inlineStr"/>
-      <c r="N71" s="5" t="inlineStr"/>
-      <c r="O71" s="5" t="inlineStr"/>
-      <c r="P71" s="5" t="inlineStr"/>
-      <c r="Q71" s="5" t="inlineStr"/>
-      <c r="R71" s="5" t="inlineStr"/>
-      <c r="S71" s="5" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="5" t="inlineStr"/>
-      <c r="B72" s="5" t="inlineStr"/>
-      <c r="C72" s="5" t="inlineStr"/>
-      <c r="D72" s="5" t="inlineStr"/>
-      <c r="E72" s="5" t="inlineStr"/>
-      <c r="F72" s="5" t="inlineStr"/>
-      <c r="G72" s="5" t="inlineStr"/>
-      <c r="H72" s="5" t="inlineStr"/>
-      <c r="I72" s="5" t="inlineStr"/>
-      <c r="J72" s="5" t="inlineStr"/>
-      <c r="K72" s="5" t="inlineStr"/>
-      <c r="L72" s="5" t="inlineStr"/>
-      <c r="M72" s="5" t="inlineStr"/>
-      <c r="N72" s="5" t="inlineStr"/>
-      <c r="O72" s="5" t="inlineStr"/>
-      <c r="P72" s="5" t="inlineStr"/>
-      <c r="Q72" s="5" t="inlineStr"/>
-      <c r="R72" s="5" t="inlineStr"/>
-      <c r="S72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr"/>
@@ -2187,192 +2208,192 @@
       <c r="R77" s="5" t="inlineStr"/>
       <c r="S77" s="5" t="inlineStr"/>
     </row>
-    <row r="78"/>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr"/>
+      <c r="B78" s="5" t="inlineStr"/>
+      <c r="C78" s="5" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr"/>
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="5" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
+      <c r="N78" s="5" t="inlineStr"/>
+      <c r="O78" s="5" t="inlineStr"/>
+      <c r="P78" s="5" t="inlineStr"/>
+      <c r="Q78" s="5" t="inlineStr"/>
+      <c r="R78" s="5" t="inlineStr"/>
+      <c r="S78" s="5" t="inlineStr"/>
+    </row>
     <row r="79">
-      <c r="A79" s="7" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr"/>
+      <c r="B79" s="5" t="inlineStr"/>
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr"/>
+      <c r="E79" s="5" t="inlineStr"/>
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr"/>
+      <c r="I79" s="5" t="inlineStr"/>
+      <c r="J79" s="5" t="inlineStr"/>
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
+      <c r="N79" s="5" t="inlineStr"/>
+      <c r="O79" s="5" t="inlineStr"/>
+      <c r="P79" s="5" t="inlineStr"/>
+      <c r="Q79" s="5" t="inlineStr"/>
+      <c r="R79" s="5" t="inlineStr"/>
+      <c r="S79" s="5" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr"/>
+      <c r="B80" s="5" t="inlineStr"/>
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr"/>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="5" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
+      <c r="N80" s="5" t="inlineStr"/>
+      <c r="O80" s="5" t="inlineStr"/>
+      <c r="P80" s="5" t="inlineStr"/>
+      <c r="Q80" s="5" t="inlineStr"/>
+      <c r="R80" s="5" t="inlineStr"/>
+      <c r="S80" s="5" t="inlineStr"/>
+    </row>
+    <row r="81"/>
+    <row r="82">
+      <c r="A82" s="7" t="inlineStr">
         <is>
           <t>增资配股</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
         <is>
           <t>是否办理
 generate</t>
         </is>
       </c>
-      <c r="B80" s="2" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>认购人
 allottee_name</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
         <is>
           <t>认购人证件/注册号
 allottee_id_number</t>
         </is>
       </c>
-      <c r="D80" s="2" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>认购人地址
 allottee_address</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>配发股数
 shares_allotted</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>股份类别
 share_class</t>
         </is>
       </c>
-      <c r="G80" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t>本次已发行股本
 issued_share_capital</t>
         </is>
       </c>
-      <c r="H80" s="2" t="inlineStr">
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>每股实缴
 amount_paid_per_share</t>
         </is>
       </c>
-      <c r="I80" s="2" t="inlineStr">
+      <c r="I83" s="2" t="inlineStr">
         <is>
           <t>本次实缴资本
 total_paid</t>
         </is>
       </c>
-      <c r="J80" s="2" t="inlineStr">
+      <c r="J83" s="2" t="inlineStr">
         <is>
           <t>币种
 currency</t>
         </is>
       </c>
-      <c r="K80" s="2" t="inlineStr">
+      <c r="K83" s="2" t="inlineStr">
         <is>
           <t>配股日期
 allotment_date</t>
         </is>
       </c>
-      <c r="L80" s="2" t="inlineStr">
+      <c r="L83" s="2" t="inlineStr">
         <is>
           <t>授权日期
 authority_date</t>
         </is>
       </c>
-      <c r="M80" s="2" t="inlineStr">
+      <c r="M83" s="2" t="inlineStr">
         <is>
           <t>是否 Form 24
 form24_required</t>
         </is>
       </c>
-      <c r="N80" s="2" t="inlineStr">
+      <c r="N83" s="2" t="inlineStr">
         <is>
           <t>证书号
 certificate_no</t>
         </is>
       </c>
-      <c r="O80" s="2" t="inlineStr">
+      <c r="O83" s="2" t="inlineStr">
         <is>
           <t>是否生成证书
 generate_certificate</t>
         </is>
       </c>
-      <c r="P80" s="2" t="inlineStr">
+      <c r="P83" s="2" t="inlineStr">
         <is>
           <t>配股后总股数
 post_allotment_total_shares</t>
         </is>
       </c>
-      <c r="Q80" s="2" t="inlineStr">
+      <c r="Q83" s="2" t="inlineStr">
         <is>
           <t>配股后已发行股本
 post_allotment_issued_share_capital</t>
         </is>
       </c>
-      <c r="R80" s="2" t="inlineStr">
+      <c r="R83" s="2" t="inlineStr">
         <is>
           <t>配股后实缴资本
 post_allotment_paid_up_capital</t>
         </is>
       </c>
-      <c r="S80" s="2" t="inlineStr">
+      <c r="S83" s="2" t="inlineStr">
         <is>
           <t>备注
 remarks</t>
         </is>
       </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="5" t="inlineStr"/>
-      <c r="B81" s="5" t="inlineStr"/>
-      <c r="C81" s="5" t="inlineStr"/>
-      <c r="D81" s="5" t="inlineStr"/>
-      <c r="E81" s="5" t="inlineStr"/>
-      <c r="F81" s="5" t="inlineStr"/>
-      <c r="G81" s="5" t="inlineStr"/>
-      <c r="H81" s="5" t="inlineStr"/>
-      <c r="I81" s="5" t="inlineStr"/>
-      <c r="J81" s="5" t="inlineStr"/>
-      <c r="K81" s="5" t="inlineStr"/>
-      <c r="L81" s="5" t="inlineStr"/>
-      <c r="M81" s="5" t="inlineStr"/>
-      <c r="N81" s="5" t="inlineStr"/>
-      <c r="O81" s="5" t="inlineStr"/>
-      <c r="P81" s="5" t="inlineStr"/>
-      <c r="Q81" s="5" t="inlineStr"/>
-      <c r="R81" s="5" t="inlineStr"/>
-      <c r="S81" s="5" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr"/>
-      <c r="B82" s="5" t="inlineStr"/>
-      <c r="C82" s="5" t="inlineStr"/>
-      <c r="D82" s="5" t="inlineStr"/>
-      <c r="E82" s="5" t="inlineStr"/>
-      <c r="F82" s="5" t="inlineStr"/>
-      <c r="G82" s="5" t="inlineStr"/>
-      <c r="H82" s="5" t="inlineStr"/>
-      <c r="I82" s="5" t="inlineStr"/>
-      <c r="J82" s="5" t="inlineStr"/>
-      <c r="K82" s="5" t="inlineStr"/>
-      <c r="L82" s="5" t="inlineStr"/>
-      <c r="M82" s="5" t="inlineStr"/>
-      <c r="N82" s="5" t="inlineStr"/>
-      <c r="O82" s="5" t="inlineStr"/>
-      <c r="P82" s="5" t="inlineStr"/>
-      <c r="Q82" s="5" t="inlineStr"/>
-      <c r="R82" s="5" t="inlineStr"/>
-      <c r="S82" s="5" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="5" t="inlineStr"/>
-      <c r="B83" s="5" t="inlineStr"/>
-      <c r="C83" s="5" t="inlineStr"/>
-      <c r="D83" s="5" t="inlineStr"/>
-      <c r="E83" s="5" t="inlineStr"/>
-      <c r="F83" s="5" t="inlineStr"/>
-      <c r="G83" s="5" t="inlineStr"/>
-      <c r="H83" s="5" t="inlineStr"/>
-      <c r="I83" s="5" t="inlineStr"/>
-      <c r="J83" s="5" t="inlineStr"/>
-      <c r="K83" s="5" t="inlineStr"/>
-      <c r="L83" s="5" t="inlineStr"/>
-      <c r="M83" s="5" t="inlineStr"/>
-      <c r="N83" s="5" t="inlineStr"/>
-      <c r="O83" s="5" t="inlineStr"/>
-      <c r="P83" s="5" t="inlineStr"/>
-      <c r="Q83" s="5" t="inlineStr"/>
-      <c r="R83" s="5" t="inlineStr"/>
-      <c r="S83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr"/>
@@ -2479,11 +2500,74 @@
       <c r="R88" s="5" t="inlineStr"/>
       <c r="S88" s="5" t="inlineStr"/>
     </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr"/>
+      <c r="B89" s="5" t="inlineStr"/>
+      <c r="C89" s="5" t="inlineStr"/>
+      <c r="D89" s="5" t="inlineStr"/>
+      <c r="E89" s="5" t="inlineStr"/>
+      <c r="F89" s="5" t="inlineStr"/>
+      <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr"/>
+      <c r="I89" s="5" t="inlineStr"/>
+      <c r="J89" s="5" t="inlineStr"/>
+      <c r="K89" s="5" t="inlineStr"/>
+      <c r="L89" s="5" t="inlineStr"/>
+      <c r="M89" s="5" t="inlineStr"/>
+      <c r="N89" s="5" t="inlineStr"/>
+      <c r="O89" s="5" t="inlineStr"/>
+      <c r="P89" s="5" t="inlineStr"/>
+      <c r="Q89" s="5" t="inlineStr"/>
+      <c r="R89" s="5" t="inlineStr"/>
+      <c r="S89" s="5" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr"/>
+      <c r="B90" s="5" t="inlineStr"/>
+      <c r="C90" s="5" t="inlineStr"/>
+      <c r="D90" s="5" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr"/>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr"/>
+      <c r="I90" s="5" t="inlineStr"/>
+      <c r="J90" s="5" t="inlineStr"/>
+      <c r="K90" s="5" t="inlineStr"/>
+      <c r="L90" s="5" t="inlineStr"/>
+      <c r="M90" s="5" t="inlineStr"/>
+      <c r="N90" s="5" t="inlineStr"/>
+      <c r="O90" s="5" t="inlineStr"/>
+      <c r="P90" s="5" t="inlineStr"/>
+      <c r="Q90" s="5" t="inlineStr"/>
+      <c r="R90" s="5" t="inlineStr"/>
+      <c r="S90" s="5" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr"/>
+      <c r="B91" s="5" t="inlineStr"/>
+      <c r="C91" s="5" t="inlineStr"/>
+      <c r="D91" s="5" t="inlineStr"/>
+      <c r="E91" s="5" t="inlineStr"/>
+      <c r="F91" s="5" t="inlineStr"/>
+      <c r="G91" s="5" t="inlineStr"/>
+      <c r="H91" s="5" t="inlineStr"/>
+      <c r="I91" s="5" t="inlineStr"/>
+      <c r="J91" s="5" t="inlineStr"/>
+      <c r="K91" s="5" t="inlineStr"/>
+      <c r="L91" s="5" t="inlineStr"/>
+      <c r="M91" s="5" t="inlineStr"/>
+      <c r="N91" s="5" t="inlineStr"/>
+      <c r="O91" s="5" t="inlineStr"/>
+      <c r="P91" s="5" t="inlineStr"/>
+      <c r="Q91" s="5" t="inlineStr"/>
+      <c r="R91" s="5" t="inlineStr"/>
+      <c r="S91" s="5" t="inlineStr"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <dataValidations count="19">
+  <dataValidations count="20">
     <dataValidation sqref="D19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
@@ -2499,46 +2583,49 @@
     <dataValidation sqref="D34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="D39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Auto,Yes,No"</formula1>
+    </dataValidation>
     <dataValidation sqref="D38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="D39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="A48:A55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A51:A58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="B48:B55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B51:B58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"appoint_director,resign_director,appoint_secretary,resign_secretary"</formula1>
     </dataValidation>
-    <dataValidation sqref="E48:E55" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E51:E58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="A59:A66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A62:A69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="C59:C66" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="C62:C69" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"ID type,ID number,Residential address,Email,Phone,Nationality,Name,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="A70:A77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A73:A80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="K70:K77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="K73:K80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"internal_paid_up_basis,acra_paid_up_capital_basis,stamp_duty_higher_of_price_or_nav"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q70:Q77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Q73:Q80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="R70:R77" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R73:R80" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="A81:A88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A84:A91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="M81:M88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M84:M91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="O81:O88" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O84:O91" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Auto,Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Default M05 director signing to all current directors
</commit_message>
<xml_diff>
--- a/templates/import/P2_maintenance_annual_blank_v7.xlsx
+++ b/templates/import/P2_maintenance_annual_blank_v7.xlsx
@@ -3165,12 +3165,12 @@
       <c r="D20" s="5" t="inlineStr"/>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>常用</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>留空默认首页董事签字人。</t>
+          <t>留空=所有当前董事，包含挂名董事；只在需要人工覆盖时填写。</t>
         </is>
       </c>
     </row>
@@ -3221,12 +3221,12 @@
       <c r="D22" s="5" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>默认董事签字人</t>
+          <t>可空</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>Annual Return 授权。</t>
+          <t>留空=第一个年审董事；只在需要指定 AR 授权人时填写。</t>
         </is>
       </c>
     </row>

</xml_diff>